<commit_message>
parts order updated with cheaper cables for ECG
</commit_message>
<xml_diff>
--- a/3_Hardware/9_Parts order form.xlsx
+++ b/3_Hardware/9_Parts order form.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bogda\Programming\PM4\PM4\3_Hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BDCB5ED-4323-4EFB-9108-76B4B2BC42BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{933BAD4D-1FC5-4170-B647-AD4177B98695}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="648" xr2:uid="{052C758A-BAC0-4DC7-8CE7-8521D951769E}"/>
   </bookViews>
@@ -20,12 +20,12 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <customWorkbookViews>
+    <customWorkbookView name="Mario Festini - Persönliche Ansicht" guid="{E7C05AF0-EEA1-11D3-A478-00D0B719A77E}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1276" windowHeight="888" tabRatio="454" activeSheetId="1"/>
+    <customWorkbookView name="Martin Studach - Persönliche Ansicht" guid="{41762A73-5BBF-11D4-A413-00D0B719978B}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1148" windowHeight="702" tabRatio="457" activeSheetId="1"/>
+    <customWorkbookView name="Werner Baumberger - Persönliche Ansicht" guid="{89927FE2-5BBA-11D4-87E4-00D0B719949C}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1276" windowHeight="908" tabRatio="457" activeSheetId="1" showStatusbar="0" showComments="commNone"/>
+    <customWorkbookView name="Patrick Mattioli - Persönliche Ansicht" guid="{D10A2CD0-5BB5-11D4-88A6-00D0B719D1AA}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1276" windowHeight="864" tabRatio="457" activeSheetId="1"/>
+    <customWorkbookView name="Patrik Jourdan - Persönliche Ansicht" guid="{ABF85D01-5BDF-11D4-A8DB-00D0B773D887}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1020" windowHeight="606" tabRatio="457" activeSheetId="1"/>
     <customWorkbookView name="mattioli - Persönliche Ansicht" guid="{6A967B41-C086-11D4-A516-00D0B719D1AA}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1276" windowHeight="890" activeSheetId="1"/>
-    <customWorkbookView name="Patrik Jourdan - Persönliche Ansicht" guid="{ABF85D01-5BDF-11D4-A8DB-00D0B773D887}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1020" windowHeight="606" tabRatio="457" activeSheetId="1"/>
-    <customWorkbookView name="Patrick Mattioli - Persönliche Ansicht" guid="{D10A2CD0-5BB5-11D4-88A6-00D0B719D1AA}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1276" windowHeight="864" tabRatio="457" activeSheetId="1"/>
-    <customWorkbookView name="Werner Baumberger - Persönliche Ansicht" guid="{89927FE2-5BBA-11D4-87E4-00D0B719949C}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1276" windowHeight="908" tabRatio="457" activeSheetId="1" showStatusbar="0" showComments="commNone"/>
-    <customWorkbookView name="Martin Studach - Persönliche Ansicht" guid="{41762A73-5BBF-11D4-A413-00D0B719978B}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1148" windowHeight="702" tabRatio="457" activeSheetId="1"/>
-    <customWorkbookView name="Mario Festini - Persönliche Ansicht" guid="{E7C05AF0-EEA1-11D3-A478-00D0B719A77E}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1276" windowHeight="888" tabRatio="454" activeSheetId="1"/>
   </customWorkbookViews>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="23">
   <si>
     <t>ArtNr.</t>
   </si>
@@ -107,22 +107,30 @@
     <t>Frontend, Herzfrequenzmesser</t>
   </si>
   <si>
-    <t>Statech systems</t>
-  </si>
-  <si>
-    <t>S2-4W-10W</t>
-  </si>
-  <si>
-    <t>Spiralkabel 2m, 4mm(w)/10mm(m), 2MΩ</t>
-  </si>
-  <si>
     <t>procamed</t>
   </si>
   <si>
-    <t>ZOLL ECG Electrodes-3 Box 10Stk</t>
+    <t xml:space="preserve">Specialised Cables EKG-EMG CABLE W/SNAP CONNECTOR </t>
   </si>
   <si>
-    <t xml:space="preserve">8900-0003 </t>
+    <t xml:space="preserve">909-SHIELD-EKGEMGPRO </t>
+  </si>
+  <si>
+    <t>8900-0003</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">ZOLL ECG Electrodes-3 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Box 10Stk</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -297,7 +305,7 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -451,13 +459,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -476,14 +480,27 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -897,26 +914,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" customFormat="1" ht="60.75" customHeight="1">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="57" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="60"/>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="61" t="s">
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="58" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="61"/>
-      <c r="K1" s="61"/>
-      <c r="L1" s="61"/>
-      <c r="M1" s="61"/>
-      <c r="N1" s="61"/>
-      <c r="O1" s="61"/>
-      <c r="P1" s="61"/>
+      <c r="F1" s="58"/>
+      <c r="G1" s="58"/>
+      <c r="H1" s="58"/>
+      <c r="I1" s="58"/>
+      <c r="J1" s="58"/>
+      <c r="K1" s="58"/>
+      <c r="L1" s="58"/>
+      <c r="M1" s="58"/>
+      <c r="N1" s="58"/>
+      <c r="O1" s="58"/>
+      <c r="P1" s="58"/>
     </row>
     <row r="2" spans="1:16" customFormat="1" ht="3" customHeight="1">
       <c r="A2" s="25"/>
@@ -990,24 +1007,24 @@
       <c r="P4" s="14"/>
     </row>
     <row r="5" spans="1:16" ht="21.75" customHeight="1">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="63" t="s">
         <v>18</v>
       </c>
-      <c r="B5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" s="2">
-        <v>6</v>
-      </c>
-      <c r="D5" s="48" t="s">
-        <v>20</v>
-      </c>
-      <c r="E5" s="6">
-        <v>12.7</v>
+      <c r="B5" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="38">
+        <v>1</v>
+      </c>
+      <c r="D5" s="47" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="24">
+        <v>9</v>
       </c>
       <c r="F5" s="31">
         <f t="shared" ref="F5:F16" si="0">C5*E5</f>
-        <v>76.199999999999989</v>
+        <v>9</v>
       </c>
       <c r="G5" s="36"/>
       <c r="H5" s="39"/>
@@ -1019,23 +1036,11 @@
     </row>
     <row r="6" spans="1:16" ht="13">
       <c r="A6" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" s="38">
-        <v>1</v>
-      </c>
-      <c r="D6" t="s">
-        <v>22</v>
-      </c>
-      <c r="E6" s="24">
         <v>9</v>
       </c>
       <c r="F6" s="31">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G6" s="36"/>
       <c r="H6" s="39"/>
@@ -1048,7 +1053,7 @@
       <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="48"/>
+      <c r="B7" s="59"/>
       <c r="D7" s="48"/>
       <c r="E7" s="24"/>
       <c r="F7" s="31">
@@ -1067,7 +1072,7 @@
       <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="48"/>
+      <c r="B8" s="59"/>
       <c r="D8" s="48"/>
       <c r="E8" s="24"/>
       <c r="F8" s="31">
@@ -1086,10 +1091,10 @@
       <c r="A9" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="48"/>
+      <c r="B9" s="59"/>
       <c r="D9" s="48"/>
       <c r="E9" s="24"/>
-      <c r="F9" s="54">
+      <c r="F9" s="52">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -1105,7 +1110,7 @@
       <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="48"/>
+      <c r="B10" s="59"/>
       <c r="C10" s="38"/>
       <c r="D10" s="48"/>
       <c r="E10" s="24"/>
@@ -1125,7 +1130,7 @@
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="48"/>
+      <c r="B11" s="59"/>
       <c r="D11" s="48"/>
       <c r="E11" s="24"/>
       <c r="F11" s="31">
@@ -1144,7 +1149,7 @@
       <c r="A12" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="48"/>
+      <c r="B12" s="59"/>
       <c r="D12"/>
       <c r="E12" s="24"/>
       <c r="F12" s="31">
@@ -1163,7 +1168,7 @@
       <c r="A13" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="48"/>
+      <c r="B13" s="59"/>
       <c r="D13"/>
       <c r="E13" s="24"/>
       <c r="F13" s="31">
@@ -1182,7 +1187,7 @@
       <c r="A14" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B14" s="48"/>
+      <c r="B14" s="59"/>
       <c r="D14"/>
       <c r="E14" s="24"/>
       <c r="F14" s="31">
@@ -1201,7 +1206,7 @@
       <c r="A15" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="48"/>
+      <c r="B15" s="59"/>
       <c r="D15"/>
       <c r="E15" s="24"/>
       <c r="F15" s="31">
@@ -1220,7 +1225,7 @@
       <c r="A16" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B16" s="48"/>
+      <c r="B16" s="59"/>
       <c r="D16"/>
       <c r="E16" s="24"/>
       <c r="F16" s="31">
@@ -1294,7 +1299,7 @@
       <c r="A20" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="B20">
+      <c r="B20" s="6">
         <v>4029748</v>
       </c>
       <c r="C20" s="38">
@@ -1320,7 +1325,7 @@
       <c r="A21" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="B21"/>
+      <c r="B21" s="6"/>
       <c r="C21" s="38"/>
       <c r="D21"/>
       <c r="E21" s="32"/>
@@ -1338,7 +1343,7 @@
       <c r="A22" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="B22" s="59"/>
+      <c r="B22" s="60"/>
       <c r="C22" s="38"/>
       <c r="D22"/>
       <c r="E22" s="32"/>
@@ -1356,7 +1361,7 @@
       <c r="A23" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="B23" s="59"/>
+      <c r="B23" s="60"/>
       <c r="D23"/>
       <c r="E23" s="32"/>
       <c r="F23" s="31">
@@ -1373,7 +1378,7 @@
       <c r="A24" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="B24" s="51"/>
+      <c r="B24" s="61"/>
       <c r="C24" s="38"/>
       <c r="D24"/>
       <c r="E24" s="32"/>
@@ -1382,7 +1387,7 @@
         <v>0</v>
       </c>
       <c r="G24" s="36"/>
-      <c r="H24" s="52"/>
+      <c r="H24" s="51"/>
       <c r="I24" s="41"/>
       <c r="J24" s="37"/>
       <c r="P24" s="46"/>
@@ -1391,7 +1396,7 @@
       <c r="A25" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="B25" s="50"/>
+      <c r="B25" s="6"/>
       <c r="C25" s="38"/>
       <c r="D25"/>
       <c r="E25" s="32"/>
@@ -1462,7 +1467,7 @@
       <c r="A29" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="B29"/>
+      <c r="B29" s="6"/>
       <c r="C29" s="38"/>
       <c r="D29" s="47"/>
       <c r="E29" s="32"/>
@@ -1627,13 +1632,21 @@
       <c r="A37" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B37"/>
-      <c r="C37" s="38"/>
-      <c r="D37"/>
-      <c r="E37" s="32"/>
+      <c r="B37" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C37" s="38">
+        <v>2</v>
+      </c>
+      <c r="D37" t="s">
+        <v>19</v>
+      </c>
+      <c r="E37" s="32">
+        <v>9.56</v>
+      </c>
       <c r="F37" s="31">
         <f t="shared" ref="F37:F61" si="2">C37*E37</f>
-        <v>0</v>
+        <v>19.12</v>
       </c>
       <c r="G37" s="36"/>
       <c r="H37" s="41"/>
@@ -1645,7 +1658,7 @@
       <c r="A38" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B38" s="51"/>
+      <c r="B38" s="61"/>
       <c r="C38" s="38"/>
       <c r="D38" s="47"/>
       <c r="E38" s="32"/>
@@ -1668,7 +1681,7 @@
       <c r="A39" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B39" s="53"/>
+      <c r="B39" s="61"/>
       <c r="C39" s="38"/>
       <c r="D39" s="47"/>
       <c r="E39" s="32"/>
@@ -1686,7 +1699,7 @@
       <c r="A40" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B40" s="50"/>
+      <c r="B40" s="6"/>
       <c r="C40" s="38"/>
       <c r="D40"/>
       <c r="E40" s="32"/>
@@ -1695,7 +1708,7 @@
         <v>0</v>
       </c>
       <c r="G40" s="36"/>
-      <c r="H40" s="52"/>
+      <c r="H40" s="51"/>
       <c r="I40" s="41"/>
       <c r="J40" s="37"/>
       <c r="P40" s="44"/>
@@ -1704,7 +1717,7 @@
       <c r="A41" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B41" s="50"/>
+      <c r="B41" s="6"/>
       <c r="C41" s="2"/>
       <c r="D41"/>
       <c r="E41" s="32"/>
@@ -1713,7 +1726,7 @@
         <v>0</v>
       </c>
       <c r="G41" s="36"/>
-      <c r="H41" s="52"/>
+      <c r="H41" s="51"/>
       <c r="I41" s="41"/>
       <c r="J41" s="37"/>
       <c r="K41" s="1"/>
@@ -1736,7 +1749,7 @@
         <v>0</v>
       </c>
       <c r="G42" s="36"/>
-      <c r="H42" s="52"/>
+      <c r="H42" s="51"/>
       <c r="I42" s="41"/>
       <c r="J42" s="37"/>
       <c r="K42" s="29"/>
@@ -1750,7 +1763,7 @@
       <c r="A43" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B43" s="50"/>
+      <c r="B43" s="6"/>
       <c r="C43" s="38"/>
       <c r="D43"/>
       <c r="E43" s="32"/>
@@ -1759,7 +1772,7 @@
         <v>0</v>
       </c>
       <c r="G43" s="36"/>
-      <c r="H43" s="52"/>
+      <c r="H43" s="51"/>
       <c r="I43" s="41"/>
       <c r="J43" s="37"/>
       <c r="K43" s="29"/>
@@ -1773,7 +1786,7 @@
       <c r="A44" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B44" s="50"/>
+      <c r="B44" s="6"/>
       <c r="C44" s="38"/>
       <c r="D44"/>
       <c r="E44" s="32"/>
@@ -1782,7 +1795,7 @@
         <v>0</v>
       </c>
       <c r="G44" s="36"/>
-      <c r="H44" s="52"/>
+      <c r="H44" s="51"/>
       <c r="I44" s="41"/>
       <c r="J44" s="37"/>
       <c r="K44" s="29"/>
@@ -1796,7 +1809,7 @@
       <c r="A45" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B45" s="50"/>
+      <c r="B45" s="6"/>
       <c r="C45" s="38"/>
       <c r="D45"/>
       <c r="E45" s="32"/>
@@ -1805,7 +1818,7 @@
         <v>0</v>
       </c>
       <c r="G45" s="36"/>
-      <c r="H45" s="52"/>
+      <c r="H45" s="51"/>
       <c r="I45" s="41"/>
       <c r="J45" s="37"/>
       <c r="K45" s="29"/>
@@ -1819,7 +1832,7 @@
       <c r="A46" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B46" s="50"/>
+      <c r="B46" s="6"/>
       <c r="D46"/>
       <c r="E46" s="32"/>
       <c r="F46" s="31">
@@ -1827,7 +1840,7 @@
         <v>0</v>
       </c>
       <c r="G46" s="36"/>
-      <c r="H46" s="52"/>
+      <c r="H46" s="51"/>
       <c r="I46" s="41"/>
       <c r="J46" s="37"/>
       <c r="P46" s="46"/>
@@ -1845,7 +1858,7 @@
         <v>0</v>
       </c>
       <c r="G47" s="36"/>
-      <c r="H47" s="52"/>
+      <c r="H47" s="51"/>
       <c r="I47" s="41"/>
       <c r="J47" s="37"/>
       <c r="K47" s="29"/>
@@ -1855,15 +1868,15 @@
       <c r="O47" s="29"/>
       <c r="P47" s="44"/>
     </row>
-    <row r="48" spans="1:16" s="56" customFormat="1" ht="13">
+    <row r="48" spans="1:16" s="54" customFormat="1" ht="13">
       <c r="A48" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B48" s="50"/>
-      <c r="C48" s="55"/>
+      <c r="B48" s="6"/>
+      <c r="C48" s="53"/>
       <c r="D48" s="50"/>
       <c r="E48" s="6"/>
-      <c r="F48" s="54">
+      <c r="F48" s="52">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -1877,11 +1890,11 @@
       <c r="A49" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B49" s="50"/>
-      <c r="C49" s="55"/>
-      <c r="D49" s="57"/>
-      <c r="E49" s="58"/>
-      <c r="F49" s="54">
+      <c r="B49" s="6"/>
+      <c r="C49" s="53"/>
+      <c r="D49" s="55"/>
+      <c r="E49" s="56"/>
+      <c r="F49" s="52">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -1889,22 +1902,22 @@
       <c r="H49" s="41"/>
       <c r="I49" s="41"/>
       <c r="J49" s="37"/>
-      <c r="K49" s="56"/>
-      <c r="L49" s="56"/>
-      <c r="M49" s="56"/>
-      <c r="N49" s="56"/>
-      <c r="O49" s="56"/>
+      <c r="K49" s="54"/>
+      <c r="L49" s="54"/>
+      <c r="M49" s="54"/>
+      <c r="N49" s="54"/>
+      <c r="O49" s="54"/>
       <c r="P49" s="46"/>
     </row>
-    <row r="50" spans="1:16" s="56" customFormat="1" ht="13">
+    <row r="50" spans="1:16" s="54" customFormat="1" ht="13">
       <c r="A50" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B50" s="50"/>
-      <c r="C50" s="55"/>
+      <c r="B50" s="6"/>
+      <c r="C50" s="53"/>
       <c r="D50" s="50"/>
-      <c r="E50" s="58"/>
-      <c r="F50" s="54">
+      <c r="E50" s="56"/>
+      <c r="F50" s="52">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -1914,15 +1927,15 @@
       <c r="J50" s="37"/>
       <c r="P50" s="34"/>
     </row>
-    <row r="51" spans="1:16" s="56" customFormat="1" ht="13">
+    <row r="51" spans="1:16" s="54" customFormat="1" ht="13">
       <c r="A51" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B51" s="50"/>
-      <c r="C51" s="55"/>
+      <c r="B51" s="6"/>
+      <c r="C51" s="53"/>
       <c r="D51" s="50"/>
-      <c r="E51" s="58"/>
-      <c r="F51" s="54">
+      <c r="E51" s="56"/>
+      <c r="F51" s="52">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -1932,15 +1945,15 @@
       <c r="J51" s="37"/>
       <c r="P51" s="44"/>
     </row>
-    <row r="52" spans="1:16" s="56" customFormat="1" ht="13">
+    <row r="52" spans="1:16" s="54" customFormat="1" ht="13">
       <c r="A52" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B52" s="50"/>
+      <c r="B52" s="6"/>
       <c r="C52" s="2"/>
       <c r="D52" s="50"/>
-      <c r="E52" s="58"/>
-      <c r="F52" s="54">
+      <c r="E52" s="56"/>
+      <c r="F52" s="52">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -1959,11 +1972,11 @@
       <c r="A53" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B53" s="50"/>
-      <c r="C53" s="55"/>
+      <c r="B53" s="6"/>
+      <c r="C53" s="53"/>
       <c r="D53" s="50"/>
-      <c r="E53" s="58"/>
-      <c r="F53" s="54">
+      <c r="E53" s="56"/>
+      <c r="F53" s="52">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -1971,41 +1984,41 @@
       <c r="H53" s="41"/>
       <c r="I53" s="41"/>
       <c r="J53" s="37"/>
-      <c r="K53" s="56"/>
-      <c r="L53" s="56"/>
-      <c r="M53" s="56"/>
-      <c r="N53" s="56"/>
-      <c r="O53" s="56"/>
+      <c r="K53" s="54"/>
+      <c r="L53" s="54"/>
+      <c r="M53" s="54"/>
+      <c r="N53" s="54"/>
+      <c r="O53" s="54"/>
       <c r="P53" s="44"/>
     </row>
     <row r="54" spans="1:16" ht="13">
       <c r="A54" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B54" s="50"/>
-      <c r="C54" s="55"/>
+      <c r="B54" s="6"/>
+      <c r="C54" s="53"/>
       <c r="D54" s="50"/>
-      <c r="E54" s="58"/>
-      <c r="F54" s="54">
+      <c r="E54" s="56"/>
+      <c r="F54" s="52">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="G54" s="36"/>
-      <c r="H54" s="52"/>
+      <c r="H54" s="51"/>
       <c r="I54" s="41"/>
       <c r="J54" s="37"/>
-      <c r="K54" s="56"/>
-      <c r="L54" s="56"/>
-      <c r="M54" s="56"/>
-      <c r="N54" s="56"/>
-      <c r="O54" s="56"/>
+      <c r="K54" s="54"/>
+      <c r="L54" s="54"/>
+      <c r="M54" s="54"/>
+      <c r="N54" s="54"/>
+      <c r="O54" s="54"/>
       <c r="P54" s="46"/>
     </row>
     <row r="55" spans="1:16" ht="13">
       <c r="A55" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B55" s="47"/>
+      <c r="B55" s="62"/>
       <c r="C55" s="38"/>
       <c r="D55" s="47"/>
       <c r="E55" s="32"/>
@@ -2014,7 +2027,7 @@
         <v>0</v>
       </c>
       <c r="G55" s="36"/>
-      <c r="H55" s="52"/>
+      <c r="H55" s="51"/>
       <c r="I55" s="41"/>
       <c r="J55" s="37"/>
       <c r="K55" s="29"/>
@@ -2226,7 +2239,7 @@
       <c r="A65" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B65"/>
+      <c r="B65" s="6"/>
       <c r="C65" s="38"/>
       <c r="D65"/>
       <c r="E65" s="6"/>
@@ -2249,7 +2262,7 @@
       <c r="A66" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B66"/>
+      <c r="B66" s="6"/>
       <c r="C66" s="38"/>
       <c r="D66" s="49"/>
       <c r="E66" s="32"/>
@@ -2335,7 +2348,7 @@
       <c r="A70" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B70"/>
+      <c r="B70" s="6"/>
       <c r="C70" s="38"/>
       <c r="D70" s="49"/>
       <c r="E70" s="32"/>

</xml_diff>

<commit_message>
disabled excel automatic backup
</commit_message>
<xml_diff>
--- a/3_Hardware/9_Parts order form.xlsx
+++ b/3_Hardware/9_Parts order form.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr date1904="1" backupFile="1" codeName="DieseArbeitsmappe" defaultThemeVersion="124226"/>
+  <workbookPr date1904="1" codeName="DieseArbeitsmappe" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bogda\Programming\PM4\PM4\3_Hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{933BAD4D-1FC5-4170-B647-AD4177B98695}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCABA9F6-A24E-4E02-94C4-5ECE7A38DA86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="648" xr2:uid="{052C758A-BAC0-4DC7-8CE7-8521D951769E}"/>
   </bookViews>
@@ -480,12 +480,6 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -501,6 +495,12 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -914,26 +914,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" customFormat="1" ht="60.75" customHeight="1">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="62" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="57"/>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
-      <c r="E1" s="58" t="s">
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="63" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="58"/>
-      <c r="G1" s="58"/>
-      <c r="H1" s="58"/>
-      <c r="I1" s="58"/>
-      <c r="J1" s="58"/>
-      <c r="K1" s="58"/>
-      <c r="L1" s="58"/>
-      <c r="M1" s="58"/>
-      <c r="N1" s="58"/>
-      <c r="O1" s="58"/>
-      <c r="P1" s="58"/>
+      <c r="F1" s="63"/>
+      <c r="G1" s="63"/>
+      <c r="H1" s="63"/>
+      <c r="I1" s="63"/>
+      <c r="J1" s="63"/>
+      <c r="K1" s="63"/>
+      <c r="L1" s="63"/>
+      <c r="M1" s="63"/>
+      <c r="N1" s="63"/>
+      <c r="O1" s="63"/>
+      <c r="P1" s="63"/>
     </row>
     <row r="2" spans="1:16" customFormat="1" ht="3" customHeight="1">
       <c r="A2" s="25"/>
@@ -1007,7 +1007,7 @@
       <c r="P4" s="14"/>
     </row>
     <row r="5" spans="1:16" ht="21.75" customHeight="1">
-      <c r="A5" s="63" t="s">
+      <c r="A5" s="61" t="s">
         <v>18</v>
       </c>
       <c r="B5" s="6" t="s">
@@ -1053,7 +1053,7 @@
       <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="59"/>
+      <c r="B7" s="57"/>
       <c r="D7" s="48"/>
       <c r="E7" s="24"/>
       <c r="F7" s="31">
@@ -1072,7 +1072,7 @@
       <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="59"/>
+      <c r="B8" s="57"/>
       <c r="D8" s="48"/>
       <c r="E8" s="24"/>
       <c r="F8" s="31">
@@ -1091,7 +1091,7 @@
       <c r="A9" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="59"/>
+      <c r="B9" s="57"/>
       <c r="D9" s="48"/>
       <c r="E9" s="24"/>
       <c r="F9" s="52">
@@ -1110,7 +1110,7 @@
       <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="59"/>
+      <c r="B10" s="57"/>
       <c r="C10" s="38"/>
       <c r="D10" s="48"/>
       <c r="E10" s="24"/>
@@ -1130,7 +1130,7 @@
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="59"/>
+      <c r="B11" s="57"/>
       <c r="D11" s="48"/>
       <c r="E11" s="24"/>
       <c r="F11" s="31">
@@ -1149,7 +1149,7 @@
       <c r="A12" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="59"/>
+      <c r="B12" s="57"/>
       <c r="D12"/>
       <c r="E12" s="24"/>
       <c r="F12" s="31">
@@ -1168,7 +1168,7 @@
       <c r="A13" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="59"/>
+      <c r="B13" s="57"/>
       <c r="D13"/>
       <c r="E13" s="24"/>
       <c r="F13" s="31">
@@ -1187,7 +1187,7 @@
       <c r="A14" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B14" s="59"/>
+      <c r="B14" s="57"/>
       <c r="D14"/>
       <c r="E14" s="24"/>
       <c r="F14" s="31">
@@ -1206,7 +1206,7 @@
       <c r="A15" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="59"/>
+      <c r="B15" s="57"/>
       <c r="D15"/>
       <c r="E15" s="24"/>
       <c r="F15" s="31">
@@ -1225,7 +1225,7 @@
       <c r="A16" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B16" s="59"/>
+      <c r="B16" s="57"/>
       <c r="D16"/>
       <c r="E16" s="24"/>
       <c r="F16" s="31">
@@ -1343,7 +1343,7 @@
       <c r="A22" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="B22" s="60"/>
+      <c r="B22" s="58"/>
       <c r="C22" s="38"/>
       <c r="D22"/>
       <c r="E22" s="32"/>
@@ -1361,7 +1361,7 @@
       <c r="A23" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="B23" s="60"/>
+      <c r="B23" s="58"/>
       <c r="D23"/>
       <c r="E23" s="32"/>
       <c r="F23" s="31">
@@ -1378,7 +1378,7 @@
       <c r="A24" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="B24" s="61"/>
+      <c r="B24" s="59"/>
       <c r="C24" s="38"/>
       <c r="D24"/>
       <c r="E24" s="32"/>
@@ -1658,7 +1658,7 @@
       <c r="A38" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B38" s="61"/>
+      <c r="B38" s="59"/>
       <c r="C38" s="38"/>
       <c r="D38" s="47"/>
       <c r="E38" s="32"/>
@@ -1681,7 +1681,7 @@
       <c r="A39" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B39" s="61"/>
+      <c r="B39" s="59"/>
       <c r="C39" s="38"/>
       <c r="D39" s="47"/>
       <c r="E39" s="32"/>
@@ -2018,7 +2018,7 @@
       <c r="A55" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B55" s="62"/>
+      <c r="B55" s="60"/>
       <c r="C55" s="38"/>
       <c r="D55" s="47"/>
       <c r="E55" s="32"/>

</xml_diff>

<commit_message>
component order form updated
</commit_message>
<xml_diff>
--- a/3_Hardware/9_Parts order form.xlsx
+++ b/3_Hardware/9_Parts order form.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bogda\Programming\PM4\PM4\3_Hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCABA9F6-A24E-4E02-94C4-5ECE7A38DA86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0B2F93A-EA6D-437F-96D2-5DB571F90696}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="648" xr2:uid="{052C758A-BAC0-4DC7-8CE7-8521D951769E}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="11370" tabRatio="648" xr2:uid="{052C758A-BAC0-4DC7-8CE7-8521D951769E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sammel Bestellungen" sheetId="7" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Sammel Bestellungen'!$1:$4,'Sammel Bestellungen'!#REF!,'Sammel Bestellungen'!$13:$19,'Sammel Bestellungen'!#REF!</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Sammel Bestellungen'!$1:$4,'Sammel Bestellungen'!#REF!,'Sammel Bestellungen'!$15:$21,'Sammel Bestellungen'!#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <customWorkbookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="23">
   <si>
     <t>ArtNr.</t>
   </si>
@@ -107,9 +107,6 @@
     <t>Frontend, Herzfrequenzmesser</t>
   </si>
   <si>
-    <t>procamed</t>
-  </si>
-  <si>
     <t xml:space="preserve">Specialised Cables EKG-EMG CABLE W/SNAP CONNECTOR </t>
   </si>
   <si>
@@ -131,6 +128,9 @@
       </rPr>
       <t>Box 10Stk</t>
     </r>
+  </si>
+  <si>
+    <t>Procamed</t>
   </si>
 </sst>
 </file>
@@ -890,7 +890,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R1805"/>
+  <dimension ref="A1:R1807"/>
   <sheetFormatPr defaultColWidth="11.54296875" defaultRowHeight="12.5" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="15.26953125" style="2" bestFit="1" customWidth="1"/>
@@ -1008,22 +1008,22 @@
     </row>
     <row r="5" spans="1:16" ht="21.75" customHeight="1">
       <c r="A5" s="61" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C5" s="38">
         <v>1</v>
       </c>
       <c r="D5" s="47" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E5" s="24">
         <v>9</v>
       </c>
       <c r="F5" s="31">
-        <f t="shared" ref="F5:F16" si="0">C5*E5</f>
+        <f t="shared" ref="F5:F18" si="0">C5*E5</f>
         <v>9</v>
       </c>
       <c r="G5" s="36"/>
@@ -1034,47 +1034,65 @@
       <c r="L5" s="9"/>
       <c r="P5" s="44"/>
     </row>
-    <row r="6" spans="1:16" ht="13">
-      <c r="A6" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F6" s="31">
-        <f t="shared" si="0"/>
+    <row r="6" spans="1:16" s="4" customFormat="1" ht="39">
+      <c r="A6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="G6" s="36"/>
-      <c r="H6" s="39"/>
-      <c r="I6" s="39"/>
-      <c r="K6" s="9"/>
-      <c r="L6" s="9"/>
-      <c r="P6" s="34"/>
-    </row>
-    <row r="7" spans="1:16" ht="13">
-      <c r="A7" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="57"/>
-      <c r="D7" s="48"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="31">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G7" s="36"/>
-      <c r="H7" s="39"/>
-      <c r="I7" s="39"/>
-      <c r="J7" s="37"/>
+      <c r="C6" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="G6" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K6" s="22"/>
+      <c r="L6" s="22"/>
+      <c r="M6" s="22"/>
+      <c r="N6" s="22"/>
+      <c r="O6" s="22"/>
+      <c r="P6" s="23" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" ht="4.5" customHeight="1">
+      <c r="A7" s="11"/>
+      <c r="B7" s="11"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="12"/>
+      <c r="E7" s="19"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="28"/>
+      <c r="H7" s="18"/>
+      <c r="I7" s="14"/>
+      <c r="J7" s="13"/>
       <c r="K7" s="9"/>
       <c r="L7" s="9"/>
-      <c r="P7" s="45"/>
+      <c r="P7" s="14"/>
     </row>
     <row r="8" spans="1:16" ht="13">
       <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="57"/>
-      <c r="D8" s="48"/>
-      <c r="E8" s="24"/>
       <c r="F8" s="31">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1082,10 +1100,9 @@
       <c r="G8" s="36"/>
       <c r="H8" s="39"/>
       <c r="I8" s="39"/>
-      <c r="J8" s="37"/>
       <c r="K8" s="9"/>
       <c r="L8" s="9"/>
-      <c r="P8" s="45"/>
+      <c r="P8" s="34"/>
     </row>
     <row r="9" spans="1:16" ht="13">
       <c r="A9" s="2" t="s">
@@ -1094,7 +1111,7 @@
       <c r="B9" s="57"/>
       <c r="D9" s="48"/>
       <c r="E9" s="24"/>
-      <c r="F9" s="52">
+      <c r="F9" s="31">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -1111,7 +1128,6 @@
         <v>9</v>
       </c>
       <c r="B10" s="57"/>
-      <c r="C10" s="38"/>
       <c r="D10" s="48"/>
       <c r="E10" s="24"/>
       <c r="F10" s="31">
@@ -1124,7 +1140,7 @@
       <c r="J10" s="37"/>
       <c r="K10" s="9"/>
       <c r="L10" s="9"/>
-      <c r="P10" s="34"/>
+      <c r="P10" s="45"/>
     </row>
     <row r="11" spans="1:16" ht="13">
       <c r="A11" s="2" t="s">
@@ -1133,7 +1149,7 @@
       <c r="B11" s="57"/>
       <c r="D11" s="48"/>
       <c r="E11" s="24"/>
-      <c r="F11" s="31">
+      <c r="F11" s="52">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -1150,7 +1166,8 @@
         <v>9</v>
       </c>
       <c r="B12" s="57"/>
-      <c r="D12"/>
+      <c r="C12" s="38"/>
+      <c r="D12" s="48"/>
       <c r="E12" s="24"/>
       <c r="F12" s="31">
         <f t="shared" si="0"/>
@@ -1162,14 +1179,14 @@
       <c r="J12" s="37"/>
       <c r="K12" s="9"/>
       <c r="L12" s="9"/>
-      <c r="P12" s="45"/>
+      <c r="P12" s="34"/>
     </row>
     <row r="13" spans="1:16" ht="13">
       <c r="A13" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B13" s="57"/>
-      <c r="D13"/>
+      <c r="D13" s="48"/>
       <c r="E13" s="24"/>
       <c r="F13" s="31">
         <f t="shared" si="0"/>
@@ -1183,7 +1200,7 @@
       <c r="L13" s="9"/>
       <c r="P13" s="45"/>
     </row>
-    <row r="14" spans="1:16" ht="13.5" customHeight="1">
+    <row r="14" spans="1:16" ht="13">
       <c r="A14" s="2" t="s">
         <v>9</v>
       </c>
@@ -1196,7 +1213,7 @@
       </c>
       <c r="G14" s="36"/>
       <c r="H14" s="39"/>
-      <c r="I14" s="40"/>
+      <c r="I14" s="39"/>
       <c r="J14" s="37"/>
       <c r="K14" s="9"/>
       <c r="L14" s="9"/>
@@ -1215,13 +1232,13 @@
       </c>
       <c r="G15" s="36"/>
       <c r="H15" s="39"/>
-      <c r="I15" s="40"/>
+      <c r="I15" s="39"/>
       <c r="J15" s="37"/>
       <c r="K15" s="9"/>
       <c r="L15" s="9"/>
       <c r="P15" s="45"/>
     </row>
-    <row r="16" spans="1:16" ht="13">
+    <row r="16" spans="1:16" ht="13.5" customHeight="1">
       <c r="A16" s="2" t="s">
         <v>9</v>
       </c>
@@ -1240,128 +1257,131 @@
       <c r="L16" s="9"/>
       <c r="P16" s="45"/>
     </row>
-    <row r="17" spans="1:16" ht="39">
-      <c r="A17" s="4" t="s">
+    <row r="17" spans="1:16" ht="13">
+      <c r="A17" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" s="57"/>
+      <c r="D17"/>
+      <c r="E17" s="24"/>
+      <c r="F17" s="31">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G17" s="36"/>
+      <c r="H17" s="39"/>
+      <c r="I17" s="40"/>
+      <c r="J17" s="37"/>
+      <c r="K17" s="9"/>
+      <c r="L17" s="9"/>
+      <c r="P17" s="45"/>
+    </row>
+    <row r="18" spans="1:16" ht="13">
+      <c r="A18" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B18" s="57"/>
+      <c r="D18"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="31">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G18" s="36"/>
+      <c r="H18" s="39"/>
+      <c r="I18" s="40"/>
+      <c r="J18" s="37"/>
+      <c r="K18" s="9"/>
+      <c r="L18" s="9"/>
+      <c r="P18" s="45"/>
+    </row>
+    <row r="19" spans="1:16" ht="39">
+      <c r="A19" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B19" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="C19" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="D19" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="E17" s="10" t="s">
+      <c r="E19" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="F17" s="10" t="s">
+      <c r="F19" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="G17" s="15" t="s">
+      <c r="G19" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="H17" s="5" t="s">
+      <c r="H19" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="I17" s="5" t="s">
+      <c r="I19" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="J17" s="5" t="s">
+      <c r="J19" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="P17" s="23" t="s">
+      <c r="P19" s="23" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="1:16" s="4" customFormat="1" ht="10">
-      <c r="A18" s="22"/>
-      <c r="B18" s="22"/>
-      <c r="C18" s="22"/>
-      <c r="D18" s="22"/>
-      <c r="E18" s="22"/>
-    </row>
-    <row r="19" spans="1:16" ht="6" customHeight="1">
-      <c r="A19" s="11"/>
-      <c r="B19" s="18"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="19"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="28"/>
-      <c r="H19" s="18"/>
-      <c r="I19" s="14"/>
-      <c r="J19" s="35"/>
-      <c r="P19" s="14"/>
-    </row>
-    <row r="20" spans="1:16" s="29" customFormat="1" ht="13">
-      <c r="A20" s="30" t="s">
-        <v>8</v>
-      </c>
-      <c r="B20" s="6">
-        <v>4029748</v>
-      </c>
-      <c r="C20" s="38">
-        <v>4</v>
-      </c>
-      <c r="D20" t="s">
-        <v>17</v>
-      </c>
-      <c r="E20" s="6">
-        <v>5.95</v>
-      </c>
-      <c r="F20" s="31">
-        <f t="shared" ref="F20:F32" si="1">C20*E20</f>
-        <v>23.8</v>
-      </c>
-      <c r="G20" s="36"/>
-      <c r="H20" s="39"/>
-      <c r="I20" s="39"/>
-      <c r="J20" s="37"/>
-      <c r="P20" s="44"/>
-    </row>
-    <row r="21" spans="1:16" s="29" customFormat="1" ht="13">
-      <c r="A21" s="30" t="s">
-        <v>8</v>
-      </c>
-      <c r="B21" s="6"/>
-      <c r="C21" s="38"/>
-      <c r="D21"/>
-      <c r="E21" s="32"/>
-      <c r="F21" s="31">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G21" s="36"/>
-      <c r="H21" s="39"/>
-      <c r="I21" s="39"/>
-      <c r="J21" s="37"/>
-      <c r="P21" s="46"/>
-    </row>
-    <row r="22" spans="1:16" s="29" customFormat="1" ht="14">
+    <row r="20" spans="1:16" s="4" customFormat="1" ht="10">
+      <c r="A20" s="22"/>
+      <c r="B20" s="22"/>
+      <c r="C20" s="22"/>
+      <c r="D20" s="22"/>
+      <c r="E20" s="22"/>
+    </row>
+    <row r="21" spans="1:16" ht="6" customHeight="1">
+      <c r="A21" s="11"/>
+      <c r="B21" s="18"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="19"/>
+      <c r="F21" s="8"/>
+      <c r="G21" s="28"/>
+      <c r="H21" s="18"/>
+      <c r="I21" s="14"/>
+      <c r="J21" s="35"/>
+      <c r="P21" s="14"/>
+    </row>
+    <row r="22" spans="1:16" s="29" customFormat="1" ht="13">
       <c r="A22" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="B22" s="58"/>
-      <c r="C22" s="38"/>
-      <c r="D22"/>
-      <c r="E22" s="32"/>
+      <c r="B22" s="6">
+        <v>4029748</v>
+      </c>
+      <c r="C22" s="38">
+        <v>4</v>
+      </c>
+      <c r="D22" t="s">
+        <v>17</v>
+      </c>
+      <c r="E22" s="6">
+        <v>5.95</v>
+      </c>
       <c r="F22" s="31">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" ref="F22:F34" si="1">C22*E22</f>
+        <v>23.8</v>
       </c>
       <c r="G22" s="36"/>
       <c r="H22" s="39"/>
       <c r="I22" s="39"/>
       <c r="J22" s="37"/>
-      <c r="P22" s="34"/>
-    </row>
-    <row r="23" spans="1:16" ht="14">
+      <c r="P22" s="44"/>
+    </row>
+    <row r="23" spans="1:16" s="29" customFormat="1" ht="13">
       <c r="A23" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="B23" s="58"/>
+      <c r="B23" s="6"/>
+      <c r="C23" s="38"/>
       <c r="D23"/>
       <c r="E23" s="32"/>
       <c r="F23" s="31">
@@ -1374,11 +1394,11 @@
       <c r="J23" s="37"/>
       <c r="P23" s="46"/>
     </row>
-    <row r="24" spans="1:16" s="29" customFormat="1" ht="13">
+    <row r="24" spans="1:16" s="29" customFormat="1" ht="14">
       <c r="A24" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="B24" s="59"/>
+      <c r="B24" s="58"/>
       <c r="C24" s="38"/>
       <c r="D24"/>
       <c r="E24" s="32"/>
@@ -1387,17 +1407,16 @@
         <v>0</v>
       </c>
       <c r="G24" s="36"/>
-      <c r="H24" s="51"/>
-      <c r="I24" s="41"/>
+      <c r="H24" s="39"/>
+      <c r="I24" s="39"/>
       <c r="J24" s="37"/>
-      <c r="P24" s="46"/>
-    </row>
-    <row r="25" spans="1:16" s="29" customFormat="1" ht="13">
+      <c r="P24" s="34"/>
+    </row>
+    <row r="25" spans="1:16" ht="14">
       <c r="A25" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="B25" s="6"/>
-      <c r="C25" s="38"/>
+      <c r="B25" s="58"/>
       <c r="D25"/>
       <c r="E25" s="32"/>
       <c r="F25" s="31">
@@ -1405,16 +1424,16 @@
         <v>0</v>
       </c>
       <c r="G25" s="36"/>
-      <c r="H25" s="41"/>
-      <c r="I25" s="41"/>
+      <c r="H25" s="39"/>
+      <c r="I25" s="39"/>
       <c r="J25" s="37"/>
-      <c r="P25" s="34"/>
+      <c r="P25" s="46"/>
     </row>
     <row r="26" spans="1:16" s="29" customFormat="1" ht="13">
       <c r="A26" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="B26" s="6"/>
+      <c r="B26" s="59"/>
       <c r="C26" s="38"/>
       <c r="D26"/>
       <c r="E26" s="32"/>
@@ -1423,16 +1442,17 @@
         <v>0</v>
       </c>
       <c r="G26" s="36"/>
-      <c r="H26" s="39"/>
+      <c r="H26" s="51"/>
       <c r="I26" s="41"/>
       <c r="J26" s="37"/>
-      <c r="P26" s="44"/>
-    </row>
-    <row r="27" spans="1:16" ht="13">
+      <c r="P26" s="46"/>
+    </row>
+    <row r="27" spans="1:16" s="29" customFormat="1" ht="13">
       <c r="A27" s="30" t="s">
         <v>8</v>
       </c>
       <c r="B27" s="6"/>
+      <c r="C27" s="38"/>
       <c r="D27"/>
       <c r="E27" s="32"/>
       <c r="F27" s="31">
@@ -1440,10 +1460,10 @@
         <v>0</v>
       </c>
       <c r="G27" s="36"/>
-      <c r="H27" s="43"/>
+      <c r="H27" s="41"/>
       <c r="I27" s="41"/>
       <c r="J27" s="37"/>
-      <c r="P27" s="46"/>
+      <c r="P27" s="34"/>
     </row>
     <row r="28" spans="1:16" s="29" customFormat="1" ht="13">
       <c r="A28" s="30" t="s">
@@ -1451,25 +1471,24 @@
       </c>
       <c r="B28" s="6"/>
       <c r="C28" s="38"/>
-      <c r="D28" s="47"/>
+      <c r="D28"/>
       <c r="E28" s="32"/>
       <c r="F28" s="31">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="G28" s="36"/>
-      <c r="H28" s="43"/>
+      <c r="H28" s="39"/>
       <c r="I28" s="41"/>
       <c r="J28" s="37"/>
       <c r="P28" s="44"/>
     </row>
-    <row r="29" spans="1:16" s="29" customFormat="1" ht="13">
+    <row r="29" spans="1:16" ht="13">
       <c r="A29" s="30" t="s">
         <v>8</v>
       </c>
       <c r="B29" s="6"/>
-      <c r="C29" s="38"/>
-      <c r="D29" s="47"/>
+      <c r="D29"/>
       <c r="E29" s="32"/>
       <c r="F29" s="31">
         <f t="shared" si="1"/>
@@ -1497,7 +1516,7 @@
       <c r="H30" s="43"/>
       <c r="I30" s="41"/>
       <c r="J30" s="37"/>
-      <c r="P30" s="34"/>
+      <c r="P30" s="44"/>
     </row>
     <row r="31" spans="1:16" s="29" customFormat="1" ht="13">
       <c r="A31" s="30" t="s">
@@ -1515,13 +1534,14 @@
       <c r="H31" s="43"/>
       <c r="I31" s="41"/>
       <c r="J31" s="37"/>
-      <c r="P31" s="44"/>
-    </row>
-    <row r="32" spans="1:16" ht="13">
+      <c r="P31" s="46"/>
+    </row>
+    <row r="32" spans="1:16" s="29" customFormat="1" ht="13">
       <c r="A32" s="30" t="s">
         <v>8</v>
       </c>
       <c r="B32" s="6"/>
+      <c r="C32" s="38"/>
       <c r="D32" s="47"/>
       <c r="E32" s="32"/>
       <c r="F32" s="31">
@@ -1532,7 +1552,7 @@
       <c r="H32" s="43"/>
       <c r="I32" s="41"/>
       <c r="J32" s="37"/>
-      <c r="P32" s="46"/>
+      <c r="P32" s="34"/>
     </row>
     <row r="33" spans="1:16" s="29" customFormat="1" ht="13">
       <c r="A33" s="30" t="s">
@@ -1543,7 +1563,7 @@
       <c r="D33" s="47"/>
       <c r="E33" s="32"/>
       <c r="F33" s="31">
-        <f>C33*E33</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="G33" s="36"/>
@@ -1552,191 +1572,185 @@
       <c r="J33" s="37"/>
       <c r="P33" s="44"/>
     </row>
-    <row r="34" spans="1:16" s="29" customFormat="1" ht="39">
-      <c r="A34" s="4" t="s">
+    <row r="34" spans="1:16" ht="13">
+      <c r="A34" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="B34" s="6"/>
+      <c r="D34" s="47"/>
+      <c r="E34" s="32"/>
+      <c r="F34" s="31">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G34" s="36"/>
+      <c r="H34" s="43"/>
+      <c r="I34" s="41"/>
+      <c r="J34" s="37"/>
+      <c r="P34" s="46"/>
+    </row>
+    <row r="35" spans="1:16" s="29" customFormat="1" ht="13">
+      <c r="A35" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="B35" s="6"/>
+      <c r="C35" s="38"/>
+      <c r="D35" s="47"/>
+      <c r="E35" s="32"/>
+      <c r="F35" s="31">
+        <f>C35*E35</f>
+        <v>0</v>
+      </c>
+      <c r="G35" s="36"/>
+      <c r="H35" s="43"/>
+      <c r="I35" s="41"/>
+      <c r="J35" s="37"/>
+      <c r="P35" s="44"/>
+    </row>
+    <row r="36" spans="1:16" s="29" customFormat="1" ht="39">
+      <c r="A36" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B34" s="10" t="s">
+      <c r="B36" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C34" s="10" t="s">
+      <c r="C36" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D34" s="10" t="s">
+      <c r="D36" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="E34" s="10" t="s">
+      <c r="E36" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="F34" s="10" t="s">
+      <c r="F36" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="G34" s="15" t="s">
+      <c r="G36" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="H34" s="5" t="s">
+      <c r="H36" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="I34" s="5" t="s">
+      <c r="I36" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="J34" s="5" t="s">
+      <c r="J36" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="K34" s="1"/>
-      <c r="L34" s="1"/>
-      <c r="M34" s="1"/>
-      <c r="N34" s="1"/>
-      <c r="O34" s="1"/>
-      <c r="P34" s="23" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="35" spans="1:16" s="29" customFormat="1">
-      <c r="A35" s="22"/>
-      <c r="B35" s="22"/>
-      <c r="C35" s="22"/>
-      <c r="D35" s="22"/>
-      <c r="E35" s="22"/>
-      <c r="F35" s="4"/>
-      <c r="G35" s="4"/>
-      <c r="H35" s="4"/>
-      <c r="I35" s="4"/>
-      <c r="J35" s="4"/>
-      <c r="K35" s="4"/>
-      <c r="L35" s="4"/>
-      <c r="M35" s="4"/>
-      <c r="N35" s="4"/>
-      <c r="O35" s="4"/>
-      <c r="P35" s="4"/>
-    </row>
-    <row r="36" spans="1:16" s="29" customFormat="1" ht="13">
-      <c r="A36" s="11"/>
-      <c r="B36" s="18"/>
-      <c r="C36" s="11"/>
-      <c r="D36" s="12"/>
-      <c r="E36" s="19"/>
-      <c r="F36" s="8"/>
-      <c r="G36" s="28"/>
-      <c r="H36" s="18"/>
-      <c r="I36" s="14"/>
-      <c r="J36" s="35"/>
       <c r="K36" s="1"/>
       <c r="L36" s="1"/>
       <c r="M36" s="1"/>
       <c r="N36" s="1"/>
       <c r="O36" s="1"/>
-      <c r="P36" s="14"/>
-    </row>
-    <row r="37" spans="1:16" s="29" customFormat="1" ht="13">
-      <c r="A37" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B37" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C37" s="38">
-        <v>2</v>
-      </c>
-      <c r="D37" t="s">
-        <v>19</v>
-      </c>
-      <c r="E37" s="32">
-        <v>9.56</v>
-      </c>
-      <c r="F37" s="31">
-        <f t="shared" ref="F37:F61" si="2">C37*E37</f>
-        <v>19.12</v>
-      </c>
-      <c r="G37" s="36"/>
-      <c r="H37" s="41"/>
-      <c r="I37" s="41"/>
-      <c r="J37" s="37"/>
-      <c r="P37" s="44"/>
-    </row>
-    <row r="38" spans="1:16" ht="13">
-      <c r="A38" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B38" s="59"/>
-      <c r="C38" s="38"/>
-      <c r="D38" s="47"/>
-      <c r="E38" s="32"/>
-      <c r="F38" s="31">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G38" s="36"/>
-      <c r="H38" s="41"/>
-      <c r="I38" s="41"/>
-      <c r="J38" s="37"/>
-      <c r="K38" s="29"/>
-      <c r="L38" s="29"/>
-      <c r="M38" s="29"/>
-      <c r="N38" s="29"/>
-      <c r="O38" s="29"/>
-      <c r="P38" s="46"/>
+      <c r="P36" s="23" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" s="29" customFormat="1">
+      <c r="A37" s="22"/>
+      <c r="B37" s="22"/>
+      <c r="C37" s="22"/>
+      <c r="D37" s="22"/>
+      <c r="E37" s="22"/>
+      <c r="F37" s="4"/>
+      <c r="G37" s="4"/>
+      <c r="H37" s="4"/>
+      <c r="I37" s="4"/>
+      <c r="J37" s="4"/>
+      <c r="K37" s="4"/>
+      <c r="L37" s="4"/>
+      <c r="M37" s="4"/>
+      <c r="N37" s="4"/>
+      <c r="O37" s="4"/>
+      <c r="P37" s="4"/>
+    </row>
+    <row r="38" spans="1:16" s="29" customFormat="1" ht="13">
+      <c r="A38" s="11"/>
+      <c r="B38" s="18"/>
+      <c r="C38" s="11"/>
+      <c r="D38" s="12"/>
+      <c r="E38" s="19"/>
+      <c r="F38" s="8"/>
+      <c r="G38" s="28"/>
+      <c r="H38" s="18"/>
+      <c r="I38" s="14"/>
+      <c r="J38" s="35"/>
+      <c r="K38" s="1"/>
+      <c r="L38" s="1"/>
+      <c r="M38" s="1"/>
+      <c r="N38" s="1"/>
+      <c r="O38" s="1"/>
+      <c r="P38" s="14"/>
     </row>
     <row r="39" spans="1:16" s="29" customFormat="1" ht="13">
       <c r="A39" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B39" s="59"/>
-      <c r="C39" s="38"/>
-      <c r="D39" s="47"/>
-      <c r="E39" s="32"/>
+      <c r="B39" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C39" s="38">
+        <v>2</v>
+      </c>
+      <c r="D39" t="s">
+        <v>18</v>
+      </c>
+      <c r="E39" s="32">
+        <v>9.56</v>
+      </c>
       <c r="F39" s="31">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f t="shared" ref="F39:F63" si="2">C39*E39</f>
+        <v>19.12</v>
       </c>
       <c r="G39" s="36"/>
       <c r="H39" s="41"/>
-      <c r="I39" s="42"/>
+      <c r="I39" s="41"/>
       <c r="J39" s="37"/>
-      <c r="P39" s="34"/>
-    </row>
-    <row r="40" spans="1:16" s="29" customFormat="1" ht="13">
+      <c r="P39" s="44"/>
+    </row>
+    <row r="40" spans="1:16" ht="13">
       <c r="A40" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B40" s="6"/>
+      <c r="B40" s="59"/>
       <c r="C40" s="38"/>
-      <c r="D40"/>
+      <c r="D40" s="47"/>
       <c r="E40" s="32"/>
       <c r="F40" s="31">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="G40" s="36"/>
-      <c r="H40" s="51"/>
+      <c r="H40" s="41"/>
       <c r="I40" s="41"/>
       <c r="J40" s="37"/>
-      <c r="P40" s="44"/>
+      <c r="K40" s="29"/>
+      <c r="L40" s="29"/>
+      <c r="M40" s="29"/>
+      <c r="N40" s="29"/>
+      <c r="O40" s="29"/>
+      <c r="P40" s="46"/>
     </row>
     <row r="41" spans="1:16" s="29" customFormat="1" ht="13">
       <c r="A41" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B41" s="6"/>
-      <c r="C41" s="2"/>
-      <c r="D41"/>
+      <c r="B41" s="59"/>
+      <c r="C41" s="38"/>
+      <c r="D41" s="47"/>
       <c r="E41" s="32"/>
       <c r="F41" s="31">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="G41" s="36"/>
-      <c r="H41" s="51"/>
-      <c r="I41" s="41"/>
+      <c r="H41" s="41"/>
+      <c r="I41" s="42"/>
       <c r="J41" s="37"/>
-      <c r="K41" s="1"/>
-      <c r="L41" s="1"/>
-      <c r="M41" s="1"/>
-      <c r="N41" s="1"/>
-      <c r="O41" s="1"/>
-      <c r="P41" s="46"/>
-    </row>
-    <row r="42" spans="1:16" ht="13">
+      <c r="P41" s="34"/>
+    </row>
+    <row r="42" spans="1:16" s="29" customFormat="1" ht="13">
       <c r="A42" s="6" t="s">
         <v>13</v>
       </c>
@@ -1752,19 +1766,14 @@
       <c r="H42" s="51"/>
       <c r="I42" s="41"/>
       <c r="J42" s="37"/>
-      <c r="K42" s="29"/>
-      <c r="L42" s="29"/>
-      <c r="M42" s="29"/>
-      <c r="N42" s="29"/>
-      <c r="O42" s="29"/>
       <c r="P42" s="44"/>
     </row>
-    <row r="43" spans="1:16" ht="13">
+    <row r="43" spans="1:16" s="29" customFormat="1" ht="13">
       <c r="A43" s="6" t="s">
         <v>13</v>
       </c>
       <c r="B43" s="6"/>
-      <c r="C43" s="38"/>
+      <c r="C43" s="2"/>
       <c r="D43"/>
       <c r="E43" s="32"/>
       <c r="F43" s="31">
@@ -1775,11 +1784,11 @@
       <c r="H43" s="51"/>
       <c r="I43" s="41"/>
       <c r="J43" s="37"/>
-      <c r="K43" s="29"/>
-      <c r="L43" s="29"/>
-      <c r="M43" s="29"/>
-      <c r="N43" s="29"/>
-      <c r="O43" s="29"/>
+      <c r="K43" s="1"/>
+      <c r="L43" s="1"/>
+      <c r="M43" s="1"/>
+      <c r="N43" s="1"/>
+      <c r="O43" s="1"/>
       <c r="P43" s="46"/>
     </row>
     <row r="44" spans="1:16" ht="13">
@@ -1803,7 +1812,7 @@
       <c r="M44" s="29"/>
       <c r="N44" s="29"/>
       <c r="O44" s="29"/>
-      <c r="P44" s="34"/>
+      <c r="P44" s="44"/>
     </row>
     <row r="45" spans="1:16" ht="13">
       <c r="A45" s="6" t="s">
@@ -1826,13 +1835,14 @@
       <c r="M45" s="29"/>
       <c r="N45" s="29"/>
       <c r="O45" s="29"/>
-      <c r="P45" s="44"/>
+      <c r="P45" s="46"/>
     </row>
     <row r="46" spans="1:16" ht="13">
       <c r="A46" s="6" t="s">
         <v>13</v>
       </c>
       <c r="B46" s="6"/>
+      <c r="C46" s="38"/>
       <c r="D46"/>
       <c r="E46" s="32"/>
       <c r="F46" s="31">
@@ -1843,7 +1853,12 @@
       <c r="H46" s="51"/>
       <c r="I46" s="41"/>
       <c r="J46" s="37"/>
-      <c r="P46" s="46"/>
+      <c r="K46" s="29"/>
+      <c r="L46" s="29"/>
+      <c r="M46" s="29"/>
+      <c r="N46" s="29"/>
+      <c r="O46" s="29"/>
+      <c r="P46" s="34"/>
     </row>
     <row r="47" spans="1:16" ht="13">
       <c r="A47" s="6" t="s">
@@ -1851,7 +1866,7 @@
       </c>
       <c r="B47" s="6"/>
       <c r="C47" s="38"/>
-      <c r="D47" s="50"/>
+      <c r="D47"/>
       <c r="E47" s="32"/>
       <c r="F47" s="31">
         <f t="shared" si="2"/>
@@ -1868,46 +1883,45 @@
       <c r="O47" s="29"/>
       <c r="P47" s="44"/>
     </row>
-    <row r="48" spans="1:16" s="54" customFormat="1" ht="13">
+    <row r="48" spans="1:16" ht="13">
       <c r="A48" s="6" t="s">
         <v>13</v>
       </c>
       <c r="B48" s="6"/>
-      <c r="C48" s="53"/>
-      <c r="D48" s="50"/>
-      <c r="E48" s="6"/>
-      <c r="F48" s="52">
+      <c r="D48"/>
+      <c r="E48" s="32"/>
+      <c r="F48" s="31">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="G48" s="36"/>
-      <c r="H48" s="41"/>
+      <c r="H48" s="51"/>
       <c r="I48" s="41"/>
       <c r="J48" s="37"/>
-      <c r="P48" s="44"/>
+      <c r="P48" s="46"/>
     </row>
     <row r="49" spans="1:16" ht="13">
       <c r="A49" s="6" t="s">
         <v>13</v>
       </c>
       <c r="B49" s="6"/>
-      <c r="C49" s="53"/>
-      <c r="D49" s="55"/>
-      <c r="E49" s="56"/>
-      <c r="F49" s="52">
+      <c r="C49" s="38"/>
+      <c r="D49" s="50"/>
+      <c r="E49" s="32"/>
+      <c r="F49" s="31">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="G49" s="36"/>
-      <c r="H49" s="41"/>
+      <c r="H49" s="51"/>
       <c r="I49" s="41"/>
       <c r="J49" s="37"/>
-      <c r="K49" s="54"/>
-      <c r="L49" s="54"/>
-      <c r="M49" s="54"/>
-      <c r="N49" s="54"/>
-      <c r="O49" s="54"/>
-      <c r="P49" s="46"/>
+      <c r="K49" s="29"/>
+      <c r="L49" s="29"/>
+      <c r="M49" s="29"/>
+      <c r="N49" s="29"/>
+      <c r="O49" s="29"/>
+      <c r="P49" s="44"/>
     </row>
     <row r="50" spans="1:16" s="54" customFormat="1" ht="13">
       <c r="A50" s="6" t="s">
@@ -1916,7 +1930,7 @@
       <c r="B50" s="6"/>
       <c r="C50" s="53"/>
       <c r="D50" s="50"/>
-      <c r="E50" s="56"/>
+      <c r="E50" s="6"/>
       <c r="F50" s="52">
         <f t="shared" si="2"/>
         <v>0</v>
@@ -1925,15 +1939,15 @@
       <c r="H50" s="41"/>
       <c r="I50" s="41"/>
       <c r="J50" s="37"/>
-      <c r="P50" s="34"/>
-    </row>
-    <row r="51" spans="1:16" s="54" customFormat="1" ht="13">
+      <c r="P50" s="44"/>
+    </row>
+    <row r="51" spans="1:16" ht="13">
       <c r="A51" s="6" t="s">
         <v>13</v>
       </c>
       <c r="B51" s="6"/>
       <c r="C51" s="53"/>
-      <c r="D51" s="50"/>
+      <c r="D51" s="55"/>
       <c r="E51" s="56"/>
       <c r="F51" s="52">
         <f t="shared" si="2"/>
@@ -1943,14 +1957,19 @@
       <c r="H51" s="41"/>
       <c r="I51" s="41"/>
       <c r="J51" s="37"/>
-      <c r="P51" s="44"/>
+      <c r="K51" s="54"/>
+      <c r="L51" s="54"/>
+      <c r="M51" s="54"/>
+      <c r="N51" s="54"/>
+      <c r="O51" s="54"/>
+      <c r="P51" s="46"/>
     </row>
     <row r="52" spans="1:16" s="54" customFormat="1" ht="13">
       <c r="A52" s="6" t="s">
         <v>13</v>
       </c>
       <c r="B52" s="6"/>
-      <c r="C52" s="2"/>
+      <c r="C52" s="53"/>
       <c r="D52" s="50"/>
       <c r="E52" s="56"/>
       <c r="F52" s="52">
@@ -1961,14 +1980,9 @@
       <c r="H52" s="41"/>
       <c r="I52" s="41"/>
       <c r="J52" s="37"/>
-      <c r="K52" s="1"/>
-      <c r="L52" s="1"/>
-      <c r="M52" s="1"/>
-      <c r="N52" s="1"/>
-      <c r="O52" s="1"/>
-      <c r="P52" s="46"/>
-    </row>
-    <row r="53" spans="1:16" ht="13">
+      <c r="P52" s="34"/>
+    </row>
+    <row r="53" spans="1:16" s="54" customFormat="1" ht="13">
       <c r="A53" s="6" t="s">
         <v>13</v>
       </c>
@@ -1984,19 +1998,14 @@
       <c r="H53" s="41"/>
       <c r="I53" s="41"/>
       <c r="J53" s="37"/>
-      <c r="K53" s="54"/>
-      <c r="L53" s="54"/>
-      <c r="M53" s="54"/>
-      <c r="N53" s="54"/>
-      <c r="O53" s="54"/>
       <c r="P53" s="44"/>
     </row>
-    <row r="54" spans="1:16" ht="13">
+    <row r="54" spans="1:16" s="54" customFormat="1" ht="13">
       <c r="A54" s="6" t="s">
         <v>13</v>
       </c>
       <c r="B54" s="6"/>
-      <c r="C54" s="53"/>
+      <c r="C54" s="2"/>
       <c r="D54" s="50"/>
       <c r="E54" s="56"/>
       <c r="F54" s="52">
@@ -2004,67 +2013,67 @@
         <v>0</v>
       </c>
       <c r="G54" s="36"/>
-      <c r="H54" s="51"/>
+      <c r="H54" s="41"/>
       <c r="I54" s="41"/>
       <c r="J54" s="37"/>
-      <c r="K54" s="54"/>
-      <c r="L54" s="54"/>
-      <c r="M54" s="54"/>
-      <c r="N54" s="54"/>
-      <c r="O54" s="54"/>
+      <c r="K54" s="1"/>
+      <c r="L54" s="1"/>
+      <c r="M54" s="1"/>
+      <c r="N54" s="1"/>
+      <c r="O54" s="1"/>
       <c r="P54" s="46"/>
     </row>
     <row r="55" spans="1:16" ht="13">
       <c r="A55" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B55" s="60"/>
-      <c r="C55" s="38"/>
-      <c r="D55" s="47"/>
-      <c r="E55" s="32"/>
-      <c r="F55" s="31">
+      <c r="B55" s="6"/>
+      <c r="C55" s="53"/>
+      <c r="D55" s="50"/>
+      <c r="E55" s="56"/>
+      <c r="F55" s="52">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="G55" s="36"/>
-      <c r="H55" s="51"/>
+      <c r="H55" s="41"/>
       <c r="I55" s="41"/>
       <c r="J55" s="37"/>
-      <c r="K55" s="29"/>
-      <c r="L55" s="29"/>
-      <c r="M55" s="29"/>
-      <c r="N55" s="29"/>
-      <c r="O55" s="29"/>
-      <c r="P55" s="46"/>
+      <c r="K55" s="54"/>
+      <c r="L55" s="54"/>
+      <c r="M55" s="54"/>
+      <c r="N55" s="54"/>
+      <c r="O55" s="54"/>
+      <c r="P55" s="44"/>
     </row>
     <row r="56" spans="1:16" ht="13">
       <c r="A56" s="6" t="s">
         <v>13</v>
       </c>
       <c r="B56" s="6"/>
-      <c r="C56" s="38"/>
-      <c r="D56" s="47"/>
-      <c r="E56" s="32"/>
-      <c r="F56" s="31">
+      <c r="C56" s="53"/>
+      <c r="D56" s="50"/>
+      <c r="E56" s="56"/>
+      <c r="F56" s="52">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="G56" s="36"/>
-      <c r="H56" s="43"/>
+      <c r="H56" s="51"/>
       <c r="I56" s="41"/>
       <c r="J56" s="37"/>
-      <c r="K56" s="29"/>
-      <c r="L56" s="29"/>
-      <c r="M56" s="29"/>
-      <c r="N56" s="29"/>
-      <c r="O56" s="29"/>
-      <c r="P56" s="34"/>
+      <c r="K56" s="54"/>
+      <c r="L56" s="54"/>
+      <c r="M56" s="54"/>
+      <c r="N56" s="54"/>
+      <c r="O56" s="54"/>
+      <c r="P56" s="46"/>
     </row>
     <row r="57" spans="1:16" ht="13">
       <c r="A57" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B57" s="6"/>
+      <c r="B57" s="60"/>
       <c r="C57" s="38"/>
       <c r="D57" s="47"/>
       <c r="E57" s="32"/>
@@ -2073,7 +2082,7 @@
         <v>0</v>
       </c>
       <c r="G57" s="36"/>
-      <c r="H57" s="43"/>
+      <c r="H57" s="51"/>
       <c r="I57" s="41"/>
       <c r="J57" s="37"/>
       <c r="K57" s="29"/>
@@ -2081,13 +2090,14 @@
       <c r="M57" s="29"/>
       <c r="N57" s="29"/>
       <c r="O57" s="29"/>
-      <c r="P57" s="44"/>
+      <c r="P57" s="46"/>
     </row>
     <row r="58" spans="1:16" ht="13">
       <c r="A58" s="6" t="s">
         <v>13</v>
       </c>
       <c r="B58" s="6"/>
+      <c r="C58" s="38"/>
       <c r="D58" s="47"/>
       <c r="E58" s="32"/>
       <c r="F58" s="31">
@@ -2098,7 +2108,12 @@
       <c r="H58" s="43"/>
       <c r="I58" s="41"/>
       <c r="J58" s="37"/>
-      <c r="P58" s="46"/>
+      <c r="K58" s="29"/>
+      <c r="L58" s="29"/>
+      <c r="M58" s="29"/>
+      <c r="N58" s="29"/>
+      <c r="O58" s="29"/>
+      <c r="P58" s="34"/>
     </row>
     <row r="59" spans="1:16" ht="13">
       <c r="A59" s="6" t="s">
@@ -2128,7 +2143,6 @@
         <v>13</v>
       </c>
       <c r="B60" s="6"/>
-      <c r="C60" s="38"/>
       <c r="D60" s="47"/>
       <c r="E60" s="32"/>
       <c r="F60" s="31">
@@ -2139,11 +2153,6 @@
       <c r="H60" s="43"/>
       <c r="I60" s="41"/>
       <c r="J60" s="37"/>
-      <c r="K60" s="29"/>
-      <c r="L60" s="29"/>
-      <c r="M60" s="29"/>
-      <c r="N60" s="29"/>
-      <c r="O60" s="29"/>
       <c r="P60" s="46"/>
     </row>
     <row r="61" spans="1:16" ht="13">
@@ -2167,119 +2176,119 @@
       <c r="M61" s="29"/>
       <c r="N61" s="29"/>
       <c r="O61" s="29"/>
-      <c r="P61" s="34"/>
-    </row>
-    <row r="62" spans="1:16" ht="39">
-      <c r="A62" s="4" t="s">
+      <c r="P61" s="44"/>
+    </row>
+    <row r="62" spans="1:16" ht="13">
+      <c r="A62" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B62" s="6"/>
+      <c r="C62" s="38"/>
+      <c r="D62" s="47"/>
+      <c r="E62" s="32"/>
+      <c r="F62" s="31">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G62" s="36"/>
+      <c r="H62" s="43"/>
+      <c r="I62" s="41"/>
+      <c r="J62" s="37"/>
+      <c r="K62" s="29"/>
+      <c r="L62" s="29"/>
+      <c r="M62" s="29"/>
+      <c r="N62" s="29"/>
+      <c r="O62" s="29"/>
+      <c r="P62" s="46"/>
+    </row>
+    <row r="63" spans="1:16" ht="13">
+      <c r="A63" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B63" s="6"/>
+      <c r="C63" s="38"/>
+      <c r="D63" s="47"/>
+      <c r="E63" s="32"/>
+      <c r="F63" s="31">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G63" s="36"/>
+      <c r="H63" s="43"/>
+      <c r="I63" s="41"/>
+      <c r="J63" s="37"/>
+      <c r="K63" s="29"/>
+      <c r="L63" s="29"/>
+      <c r="M63" s="29"/>
+      <c r="N63" s="29"/>
+      <c r="O63" s="29"/>
+      <c r="P63" s="34"/>
+    </row>
+    <row r="64" spans="1:16" ht="39">
+      <c r="A64" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B62" s="10" t="s">
+      <c r="B64" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C62" s="10" t="s">
+      <c r="C64" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D62" s="10" t="s">
+      <c r="D64" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="E62" s="10" t="s">
+      <c r="E64" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="F62" s="10" t="s">
+      <c r="F64" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="G62" s="15" t="s">
+      <c r="G64" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="H62" s="5" t="s">
+      <c r="H64" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="I62" s="5" t="s">
+      <c r="I64" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="J62" s="5" t="s">
+      <c r="J64" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="P62" s="23" t="s">
+      <c r="P64" s="23" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="63" spans="1:16">
-      <c r="A63" s="22"/>
-      <c r="B63" s="22"/>
-      <c r="C63" s="22"/>
-      <c r="D63" s="22"/>
-      <c r="E63" s="22"/>
-      <c r="F63" s="4"/>
-      <c r="G63" s="4"/>
-      <c r="H63" s="4"/>
-      <c r="I63" s="4"/>
-      <c r="J63" s="4"/>
-      <c r="K63" s="4"/>
-      <c r="L63" s="4"/>
-      <c r="M63" s="4"/>
-      <c r="N63" s="4"/>
-      <c r="O63" s="4"/>
-      <c r="P63" s="4"/>
-    </row>
-    <row r="64" spans="1:16" ht="13">
-      <c r="A64" s="11"/>
-      <c r="B64" s="18"/>
-      <c r="C64" s="11"/>
-      <c r="D64" s="12"/>
-      <c r="E64" s="19"/>
-      <c r="F64" s="8"/>
-      <c r="G64" s="28"/>
-      <c r="H64" s="18"/>
-      <c r="I64" s="14"/>
-      <c r="J64" s="35"/>
-      <c r="P64" s="14"/>
-    </row>
-    <row r="65" spans="1:16" ht="13">
-      <c r="A65" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B65" s="6"/>
-      <c r="C65" s="38"/>
-      <c r="D65"/>
-      <c r="E65" s="6"/>
-      <c r="F65" s="31">
-        <f t="shared" ref="F65:F85" si="3">C65*E65</f>
-        <v>0</v>
-      </c>
-      <c r="G65" s="36"/>
-      <c r="H65" s="41"/>
-      <c r="I65" s="41"/>
-      <c r="J65" s="37"/>
-      <c r="K65" s="29"/>
-      <c r="L65" s="29"/>
-      <c r="M65" s="29"/>
-      <c r="N65" s="29"/>
-      <c r="O65" s="29"/>
-      <c r="P65" s="44"/>
+    <row r="65" spans="1:16">
+      <c r="A65" s="22"/>
+      <c r="B65" s="22"/>
+      <c r="C65" s="22"/>
+      <c r="D65" s="22"/>
+      <c r="E65" s="22"/>
+      <c r="F65" s="4"/>
+      <c r="G65" s="4"/>
+      <c r="H65" s="4"/>
+      <c r="I65" s="4"/>
+      <c r="J65" s="4"/>
+      <c r="K65" s="4"/>
+      <c r="L65" s="4"/>
+      <c r="M65" s="4"/>
+      <c r="N65" s="4"/>
+      <c r="O65" s="4"/>
+      <c r="P65" s="4"/>
     </row>
     <row r="66" spans="1:16" ht="13">
-      <c r="A66" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B66" s="6"/>
-      <c r="C66" s="38"/>
-      <c r="D66" s="49"/>
-      <c r="E66" s="32"/>
-      <c r="F66" s="31">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G66" s="36"/>
-      <c r="H66" s="41"/>
-      <c r="I66" s="41"/>
-      <c r="J66" s="37"/>
-      <c r="K66" s="29"/>
-      <c r="L66" s="29"/>
-      <c r="M66" s="29"/>
-      <c r="N66" s="29"/>
-      <c r="O66" s="29"/>
-      <c r="P66" s="46"/>
+      <c r="A66" s="11"/>
+      <c r="B66" s="18"/>
+      <c r="C66" s="11"/>
+      <c r="D66" s="12"/>
+      <c r="E66" s="19"/>
+      <c r="F66" s="8"/>
+      <c r="G66" s="28"/>
+      <c r="H66" s="18"/>
+      <c r="I66" s="14"/>
+      <c r="J66" s="35"/>
+      <c r="P66" s="14"/>
     </row>
     <row r="67" spans="1:16" ht="13">
       <c r="A67" s="6" t="s">
@@ -2288,9 +2297,9 @@
       <c r="B67" s="6"/>
       <c r="C67" s="38"/>
       <c r="D67"/>
-      <c r="E67" s="32"/>
+      <c r="E67" s="6"/>
       <c r="F67" s="31">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="F67:F87" si="3">C67*E67</f>
         <v>0</v>
       </c>
       <c r="G67" s="36"/>
@@ -2302,7 +2311,7 @@
       <c r="M67" s="29"/>
       <c r="N67" s="29"/>
       <c r="O67" s="29"/>
-      <c r="P67" s="34"/>
+      <c r="P67" s="44"/>
     </row>
     <row r="68" spans="1:16" ht="13">
       <c r="A68" s="6" t="s">
@@ -2310,7 +2319,7 @@
       </c>
       <c r="B68" s="6"/>
       <c r="C68" s="38"/>
-      <c r="D68"/>
+      <c r="D68" s="49"/>
       <c r="E68" s="32"/>
       <c r="F68" s="31">
         <f t="shared" si="3"/>
@@ -2325,13 +2334,14 @@
       <c r="M68" s="29"/>
       <c r="N68" s="29"/>
       <c r="O68" s="29"/>
-      <c r="P68" s="44"/>
+      <c r="P68" s="46"/>
     </row>
     <row r="69" spans="1:16" ht="13">
       <c r="A69" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B69" s="6"/>
+      <c r="C69" s="38"/>
       <c r="D69"/>
       <c r="E69" s="32"/>
       <c r="F69" s="31">
@@ -2342,7 +2352,12 @@
       <c r="H69" s="41"/>
       <c r="I69" s="41"/>
       <c r="J69" s="37"/>
-      <c r="P69" s="46"/>
+      <c r="K69" s="29"/>
+      <c r="L69" s="29"/>
+      <c r="M69" s="29"/>
+      <c r="N69" s="29"/>
+      <c r="O69" s="29"/>
+      <c r="P69" s="34"/>
     </row>
     <row r="70" spans="1:16" ht="13">
       <c r="A70" s="6" t="s">
@@ -2350,14 +2365,14 @@
       </c>
       <c r="B70" s="6"/>
       <c r="C70" s="38"/>
-      <c r="D70" s="49"/>
+      <c r="D70"/>
       <c r="E70" s="32"/>
       <c r="F70" s="31">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="G70" s="36"/>
-      <c r="H70" s="43"/>
+      <c r="H70" s="41"/>
       <c r="I70" s="41"/>
       <c r="J70" s="37"/>
       <c r="K70" s="29"/>
@@ -2372,7 +2387,6 @@
         <v>15</v>
       </c>
       <c r="B71" s="6"/>
-      <c r="C71" s="38"/>
       <c r="D71"/>
       <c r="E71" s="32"/>
       <c r="F71" s="31">
@@ -2380,14 +2394,9 @@
         <v>0</v>
       </c>
       <c r="G71" s="36"/>
-      <c r="H71" s="43"/>
+      <c r="H71" s="41"/>
       <c r="I71" s="41"/>
       <c r="J71" s="37"/>
-      <c r="K71" s="29"/>
-      <c r="L71" s="29"/>
-      <c r="M71" s="29"/>
-      <c r="N71" s="29"/>
-      <c r="O71" s="29"/>
       <c r="P71" s="46"/>
     </row>
     <row r="72" spans="1:16" ht="13">
@@ -2396,7 +2405,7 @@
       </c>
       <c r="B72" s="6"/>
       <c r="C72" s="38"/>
-      <c r="D72"/>
+      <c r="D72" s="49"/>
       <c r="E72" s="32"/>
       <c r="F72" s="31">
         <f t="shared" si="3"/>
@@ -2411,7 +2420,7 @@
       <c r="M72" s="29"/>
       <c r="N72" s="29"/>
       <c r="O72" s="29"/>
-      <c r="P72" s="34"/>
+      <c r="P72" s="44"/>
     </row>
     <row r="73" spans="1:16" ht="13">
       <c r="A73" s="6" t="s">
@@ -2434,13 +2443,14 @@
       <c r="M73" s="29"/>
       <c r="N73" s="29"/>
       <c r="O73" s="29"/>
-      <c r="P73" s="44"/>
+      <c r="P73" s="46"/>
     </row>
     <row r="74" spans="1:16" ht="13">
       <c r="A74" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B74" s="6"/>
+      <c r="C74" s="38"/>
       <c r="D74"/>
       <c r="E74" s="32"/>
       <c r="F74" s="31">
@@ -2451,7 +2461,12 @@
       <c r="H74" s="43"/>
       <c r="I74" s="41"/>
       <c r="J74" s="37"/>
-      <c r="P74" s="46"/>
+      <c r="K74" s="29"/>
+      <c r="L74" s="29"/>
+      <c r="M74" s="29"/>
+      <c r="N74" s="29"/>
+      <c r="O74" s="29"/>
+      <c r="P74" s="34"/>
     </row>
     <row r="75" spans="1:16" ht="13">
       <c r="A75" s="6" t="s">
@@ -2459,7 +2474,7 @@
       </c>
       <c r="B75" s="6"/>
       <c r="C75" s="38"/>
-      <c r="D75" s="47"/>
+      <c r="D75"/>
       <c r="E75" s="32"/>
       <c r="F75" s="31">
         <f t="shared" si="3"/>
@@ -2481,8 +2496,7 @@
         <v>15</v>
       </c>
       <c r="B76" s="6"/>
-      <c r="C76" s="38"/>
-      <c r="D76" s="47"/>
+      <c r="D76"/>
       <c r="E76" s="32"/>
       <c r="F76" s="31">
         <f t="shared" si="3"/>
@@ -2492,11 +2506,6 @@
       <c r="H76" s="43"/>
       <c r="I76" s="41"/>
       <c r="J76" s="37"/>
-      <c r="K76" s="29"/>
-      <c r="L76" s="29"/>
-      <c r="M76" s="29"/>
-      <c r="N76" s="29"/>
-      <c r="O76" s="29"/>
       <c r="P76" s="46"/>
     </row>
     <row r="77" spans="1:16" ht="13">
@@ -2520,7 +2529,7 @@
       <c r="M77" s="29"/>
       <c r="N77" s="29"/>
       <c r="O77" s="29"/>
-      <c r="P77" s="34"/>
+      <c r="P77" s="44"/>
     </row>
     <row r="78" spans="1:16" ht="13">
       <c r="A78" s="6" t="s">
@@ -2543,13 +2552,14 @@
       <c r="M78" s="29"/>
       <c r="N78" s="29"/>
       <c r="O78" s="29"/>
-      <c r="P78" s="44"/>
+      <c r="P78" s="46"/>
     </row>
     <row r="79" spans="1:16" ht="13">
       <c r="A79" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B79" s="6"/>
+      <c r="C79" s="38"/>
       <c r="D79" s="47"/>
       <c r="E79" s="32"/>
       <c r="F79" s="31">
@@ -2560,7 +2570,12 @@
       <c r="H79" s="43"/>
       <c r="I79" s="41"/>
       <c r="J79" s="37"/>
-      <c r="P79" s="46"/>
+      <c r="K79" s="29"/>
+      <c r="L79" s="29"/>
+      <c r="M79" s="29"/>
+      <c r="N79" s="29"/>
+      <c r="O79" s="29"/>
+      <c r="P79" s="34"/>
     </row>
     <row r="80" spans="1:16" ht="13">
       <c r="A80" s="6" t="s">
@@ -2590,7 +2605,6 @@
         <v>15</v>
       </c>
       <c r="B81" s="6"/>
-      <c r="C81" s="38"/>
       <c r="D81" s="47"/>
       <c r="E81" s="32"/>
       <c r="F81" s="31">
@@ -2601,11 +2615,6 @@
       <c r="H81" s="43"/>
       <c r="I81" s="41"/>
       <c r="J81" s="37"/>
-      <c r="K81" s="29"/>
-      <c r="L81" s="29"/>
-      <c r="M81" s="29"/>
-      <c r="N81" s="29"/>
-      <c r="O81" s="29"/>
       <c r="P81" s="46"/>
     </row>
     <row r="82" spans="1:16" ht="13">
@@ -2629,7 +2638,7 @@
       <c r="M82" s="29"/>
       <c r="N82" s="29"/>
       <c r="O82" s="29"/>
-      <c r="P82" s="34"/>
+      <c r="P82" s="44"/>
     </row>
     <row r="83" spans="1:16" ht="13">
       <c r="A83" s="6" t="s">
@@ -2652,7 +2661,7 @@
       <c r="M83" s="29"/>
       <c r="N83" s="29"/>
       <c r="O83" s="29"/>
-      <c r="P83" s="44"/>
+      <c r="P83" s="46"/>
     </row>
     <row r="84" spans="1:16" ht="13">
       <c r="A84" s="6" t="s">
@@ -2675,13 +2684,14 @@
       <c r="M84" s="29"/>
       <c r="N84" s="29"/>
       <c r="O84" s="29"/>
-      <c r="P84" s="44"/>
+      <c r="P84" s="34"/>
     </row>
     <row r="85" spans="1:16" ht="13">
       <c r="A85" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B85" s="6"/>
+      <c r="C85" s="38"/>
       <c r="D85" s="47"/>
       <c r="E85" s="32"/>
       <c r="F85" s="31">
@@ -2692,13 +2702,52 @@
       <c r="H85" s="43"/>
       <c r="I85" s="41"/>
       <c r="J85" s="37"/>
-      <c r="P85" s="46"/>
-    </row>
-    <row r="86" spans="1:16">
-      <c r="F86" s="16"/>
-    </row>
-    <row r="87" spans="1:16">
-      <c r="F87" s="16"/>
+      <c r="K85" s="29"/>
+      <c r="L85" s="29"/>
+      <c r="M85" s="29"/>
+      <c r="N85" s="29"/>
+      <c r="O85" s="29"/>
+      <c r="P85" s="44"/>
+    </row>
+    <row r="86" spans="1:16" ht="13">
+      <c r="A86" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B86" s="6"/>
+      <c r="C86" s="38"/>
+      <c r="D86" s="47"/>
+      <c r="E86" s="32"/>
+      <c r="F86" s="31">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="G86" s="36"/>
+      <c r="H86" s="43"/>
+      <c r="I86" s="41"/>
+      <c r="J86" s="37"/>
+      <c r="K86" s="29"/>
+      <c r="L86" s="29"/>
+      <c r="M86" s="29"/>
+      <c r="N86" s="29"/>
+      <c r="O86" s="29"/>
+      <c r="P86" s="44"/>
+    </row>
+    <row r="87" spans="1:16" ht="13">
+      <c r="A87" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B87" s="6"/>
+      <c r="D87" s="47"/>
+      <c r="E87" s="32"/>
+      <c r="F87" s="31">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="G87" s="36"/>
+      <c r="H87" s="43"/>
+      <c r="I87" s="41"/>
+      <c r="J87" s="37"/>
+      <c r="P87" s="46"/>
     </row>
     <row r="88" spans="1:16">
       <c r="F88" s="16"/>
@@ -7853,6 +7902,12 @@
     </row>
     <row r="1805" spans="6:6">
       <c r="F1805" s="16"/>
+    </row>
+    <row r="1806" spans="6:6">
+      <c r="F1806" s="16"/>
+    </row>
+    <row r="1807" spans="6:6">
+      <c r="F1807" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
component order form (capacitors) + bom
</commit_message>
<xml_diff>
--- a/3_Hardware/9_Parts order form.xlsx
+++ b/3_Hardware/9_Parts order form.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bogda\Programming\PM4\PM4\3_Hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0B2F93A-EA6D-437F-96D2-5DB571F90696}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2139B156-0CFB-4712-B2D5-B353279DA633}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="11370" tabRatio="648" xr2:uid="{052C758A-BAC0-4DC7-8CE7-8521D951769E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="648" xr2:uid="{052C758A-BAC0-4DC7-8CE7-8521D951769E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sammel Bestellungen" sheetId="7" r:id="rId1"/>
@@ -20,12 +20,12 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <customWorkbookViews>
+    <customWorkbookView name="mattioli - Persönliche Ansicht" guid="{6A967B41-C086-11D4-A516-00D0B719D1AA}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1276" windowHeight="890" activeSheetId="1"/>
+    <customWorkbookView name="Patrik Jourdan - Persönliche Ansicht" guid="{ABF85D01-5BDF-11D4-A8DB-00D0B773D887}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1020" windowHeight="606" tabRatio="457" activeSheetId="1"/>
+    <customWorkbookView name="Patrick Mattioli - Persönliche Ansicht" guid="{D10A2CD0-5BB5-11D4-88A6-00D0B719D1AA}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1276" windowHeight="864" tabRatio="457" activeSheetId="1"/>
+    <customWorkbookView name="Werner Baumberger - Persönliche Ansicht" guid="{89927FE2-5BBA-11D4-87E4-00D0B719949C}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1276" windowHeight="908" tabRatio="457" activeSheetId="1" showStatusbar="0" showComments="commNone"/>
+    <customWorkbookView name="Martin Studach - Persönliche Ansicht" guid="{41762A73-5BBF-11D4-A413-00D0B719978B}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1148" windowHeight="702" tabRatio="457" activeSheetId="1"/>
     <customWorkbookView name="Mario Festini - Persönliche Ansicht" guid="{E7C05AF0-EEA1-11D3-A478-00D0B719A77E}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1276" windowHeight="888" tabRatio="454" activeSheetId="1"/>
-    <customWorkbookView name="Martin Studach - Persönliche Ansicht" guid="{41762A73-5BBF-11D4-A413-00D0B719978B}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1148" windowHeight="702" tabRatio="457" activeSheetId="1"/>
-    <customWorkbookView name="Werner Baumberger - Persönliche Ansicht" guid="{89927FE2-5BBA-11D4-87E4-00D0B719949C}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1276" windowHeight="908" tabRatio="457" activeSheetId="1" showStatusbar="0" showComments="commNone"/>
-    <customWorkbookView name="Patrick Mattioli - Persönliche Ansicht" guid="{D10A2CD0-5BB5-11D4-88A6-00D0B719D1AA}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1276" windowHeight="864" tabRatio="457" activeSheetId="1"/>
-    <customWorkbookView name="Patrik Jourdan - Persönliche Ansicht" guid="{ABF85D01-5BDF-11D4-A8DB-00D0B773D887}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1020" windowHeight="606" tabRatio="457" activeSheetId="1"/>
-    <customWorkbookView name="mattioli - Persönliche Ansicht" guid="{6A967B41-C086-11D4-A516-00D0B719D1AA}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1276" windowHeight="890" activeSheetId="1"/>
   </customWorkbookViews>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="42">
   <si>
     <t>ArtNr.</t>
   </si>
@@ -104,9 +104,6 @@
  (Distrelec, Farnell, Mouser), Einreichen bis Montag Abend</t>
   </si>
   <si>
-    <t>Frontend, Herzfrequenzmesser</t>
-  </si>
-  <si>
     <t xml:space="preserve">Specialised Cables EKG-EMG CABLE W/SNAP CONNECTOR </t>
   </si>
   <si>
@@ -132,6 +129,66 @@
   <si>
     <t>Procamed</t>
   </si>
+  <si>
+    <t>C0603C104K5RACAUTO</t>
+  </si>
+  <si>
+    <t>Keramikvielschichtkondensator, SMD, AEC-Q200, 0.1 µF, 50 V, 0603 [Metrisch 1608], ± 10%, X7R</t>
+  </si>
+  <si>
+    <t>C1608X5R1A106K080AC</t>
+  </si>
+  <si>
+    <t>Keramikvielschichtkondensator, SMD, 10 µF, 10 V, 0603 [Metrisch 1608], ± 10%, X5R</t>
+  </si>
+  <si>
+    <t>C0603S472K5RACAUTO</t>
+  </si>
+  <si>
+    <t>Keramikvielschichtkondensator, SMD, 4700 pF, 50 V, 0603 [Metrisch 1608], ± 10%, X7R</t>
+  </si>
+  <si>
+    <t>CC0805KKX6S5BB106</t>
+  </si>
+  <si>
+    <t>Keramikvielschichtkondensator, SMD, 10 µF, 6.3 V, 0805 [Metrisch 2012], ± 10%, X6S</t>
+  </si>
+  <si>
+    <t>Keramikvielschichtkondensator, SMD, 0.1 µF, 50 V, 0805 [Metrisch 2012], ± 10%, X7R</t>
+  </si>
+  <si>
+    <t>0805B104K500CT</t>
+  </si>
+  <si>
+    <t>Keramikvielschichtkondensator, SMD, 0.33 µF, 10 V, 0603 [Metrisch 1608], ± 10%, X7R</t>
+  </si>
+  <si>
+    <t>Frontend, Herzfrequenzmesser, 2 bis 3.5V, -40 bis 85°C, LFCSP-EP-20</t>
+  </si>
+  <si>
+    <t>GRM31CR60J107KEA8K</t>
+  </si>
+  <si>
+    <t>Keramikvielschichtkondensator, SMD, 100 µF, 6.3 V, 1206 [Metrisch 3216], ± 10%, X5R</t>
+  </si>
+  <si>
+    <t>C0603C152J1RACTU</t>
+  </si>
+  <si>
+    <t>Keramikvielschichtkondensator, SMD, 1500 pF, 100 V, 0603 [Metrisch 1608], ± 5%, X7R</t>
+  </si>
+  <si>
+    <t>0603B102K500CT</t>
+  </si>
+  <si>
+    <t>Keramikvielschichtkondensator, SMD, 1000 pF, 50 V, 0603 [Metrisch 1608], ± 10%, X7R</t>
+  </si>
+  <si>
+    <t>C0603C103K5RACTU</t>
+  </si>
+  <si>
+    <t>Keramikvielschichtkondensator, SMD, 0.01 µF, 50 V, 0603 [Metrisch 1608], ± 10%, X7R</t>
+  </si>
 </sst>
 </file>
 
@@ -142,7 +199,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.00_ ;[Red]\-#,##0.00\ "/>
     <numFmt numFmtId="166" formatCode="##\ ##\ ##"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="20">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -245,11 +302,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="11"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
@@ -303,9 +355,9 @@
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -452,7 +504,7 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -480,13 +532,10 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -914,26 +963,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" customFormat="1" ht="60.75" customHeight="1">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="61" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="63" t="s">
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="62" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="63"/>
-      <c r="G1" s="63"/>
-      <c r="H1" s="63"/>
-      <c r="I1" s="63"/>
-      <c r="J1" s="63"/>
-      <c r="K1" s="63"/>
-      <c r="L1" s="63"/>
-      <c r="M1" s="63"/>
-      <c r="N1" s="63"/>
-      <c r="O1" s="63"/>
-      <c r="P1" s="63"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
+      <c r="L1" s="62"/>
+      <c r="M1" s="62"/>
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
     </row>
     <row r="2" spans="1:16" customFormat="1" ht="3" customHeight="1">
       <c r="A2" s="25"/>
@@ -1007,17 +1056,17 @@
       <c r="P4" s="14"/>
     </row>
     <row r="5" spans="1:16" ht="21.75" customHeight="1">
-      <c r="A5" s="61" t="s">
-        <v>22</v>
+      <c r="A5" s="60" t="s">
+        <v>21</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C5" s="38">
         <v>1</v>
       </c>
       <c r="D5" s="47" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E5" s="24">
         <v>9</v>
@@ -1361,7 +1410,7 @@
         <v>4</v>
       </c>
       <c r="D22" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="E22" s="6">
         <v>5.95</v>
@@ -1380,13 +1429,21 @@
       <c r="A23" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="B23" s="6"/>
-      <c r="C23" s="38"/>
-      <c r="D23"/>
-      <c r="E23" s="32"/>
+      <c r="B23" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C23" s="38">
+        <v>21</v>
+      </c>
+      <c r="D23" t="s">
+        <v>23</v>
+      </c>
+      <c r="E23" s="32">
+        <v>3.9100000000000003E-2</v>
+      </c>
       <c r="F23" s="31">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.82110000000000005</v>
       </c>
       <c r="G23" s="36"/>
       <c r="H23" s="39"/>
@@ -1394,17 +1451,25 @@
       <c r="J23" s="37"/>
       <c r="P23" s="46"/>
     </row>
-    <row r="24" spans="1:16" s="29" customFormat="1" ht="14">
+    <row r="24" spans="1:16" s="29" customFormat="1" ht="13">
       <c r="A24" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="B24" s="58"/>
-      <c r="C24" s="38"/>
-      <c r="D24"/>
-      <c r="E24" s="32"/>
+      <c r="B24" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C24" s="38">
+        <v>18</v>
+      </c>
+      <c r="D24" t="s">
+        <v>25</v>
+      </c>
+      <c r="E24" s="32">
+        <v>8.8300000000000003E-2</v>
+      </c>
       <c r="F24" s="31">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1.5894000000000001</v>
       </c>
       <c r="G24" s="36"/>
       <c r="H24" s="39"/>
@@ -1412,16 +1477,25 @@
       <c r="J24" s="37"/>
       <c r="P24" s="34"/>
     </row>
-    <row r="25" spans="1:16" ht="14">
+    <row r="25" spans="1:16" ht="13">
       <c r="A25" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="B25" s="58"/>
-      <c r="D25"/>
-      <c r="E25" s="32"/>
+      <c r="B25" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C25" s="2">
+        <v>12</v>
+      </c>
+      <c r="D25" t="s">
+        <v>35</v>
+      </c>
+      <c r="E25" s="32">
+        <v>0.224</v>
+      </c>
       <c r="F25" s="31">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2.6880000000000002</v>
       </c>
       <c r="G25" s="36"/>
       <c r="H25" s="39"/>
@@ -1433,13 +1507,21 @@
       <c r="A26" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="B26" s="59"/>
-      <c r="C26" s="38"/>
-      <c r="D26"/>
-      <c r="E26" s="32"/>
+      <c r="B26" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C26" s="38">
+        <v>12</v>
+      </c>
+      <c r="D26" t="s">
+        <v>27</v>
+      </c>
+      <c r="E26" s="32">
+        <v>0.10100000000000001</v>
+      </c>
       <c r="F26" s="31">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1.2120000000000002</v>
       </c>
       <c r="G26" s="36"/>
       <c r="H26" s="51"/>
@@ -1451,13 +1533,21 @@
       <c r="A27" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="B27" s="6"/>
-      <c r="C27" s="38"/>
-      <c r="D27"/>
-      <c r="E27" s="32"/>
+      <c r="B27" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C27" s="38">
+        <v>6</v>
+      </c>
+      <c r="D27" t="s">
+        <v>29</v>
+      </c>
+      <c r="E27" s="32">
+        <v>9.4E-2</v>
+      </c>
       <c r="F27" s="31">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.56400000000000006</v>
       </c>
       <c r="G27" s="36"/>
       <c r="H27" s="41"/>
@@ -1469,13 +1559,21 @@
       <c r="A28" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="B28" s="6"/>
-      <c r="C28" s="38"/>
-      <c r="D28"/>
-      <c r="E28" s="32"/>
+      <c r="B28" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C28" s="38">
+        <v>6</v>
+      </c>
+      <c r="D28" t="s">
+        <v>30</v>
+      </c>
+      <c r="E28" s="32">
+        <v>1.35E-2</v>
+      </c>
       <c r="F28" s="31">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>8.1000000000000003E-2</v>
       </c>
       <c r="G28" s="36"/>
       <c r="H28" s="39"/>
@@ -1487,12 +1585,21 @@
       <c r="A29" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="B29" s="6"/>
-      <c r="D29"/>
-      <c r="E29" s="32"/>
+      <c r="B29" s="6">
+        <v>885012206023</v>
+      </c>
+      <c r="C29" s="2">
+        <v>6</v>
+      </c>
+      <c r="D29" t="s">
+        <v>32</v>
+      </c>
+      <c r="E29" s="32">
+        <v>6.2300000000000001E-2</v>
+      </c>
       <c r="F29" s="31">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.37380000000000002</v>
       </c>
       <c r="G29" s="36"/>
       <c r="H29" s="43"/>
@@ -1504,13 +1611,21 @@
       <c r="A30" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="B30" s="6"/>
-      <c r="C30" s="38"/>
-      <c r="D30" s="47"/>
-      <c r="E30" s="32"/>
+      <c r="B30" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C30" s="38">
+        <v>3</v>
+      </c>
+      <c r="D30" s="47" t="s">
+        <v>37</v>
+      </c>
+      <c r="E30" s="32">
+        <v>0.14099999999999999</v>
+      </c>
       <c r="F30" s="31">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.42299999999999993</v>
       </c>
       <c r="G30" s="36"/>
       <c r="H30" s="43"/>
@@ -1522,13 +1637,21 @@
       <c r="A31" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="B31" s="6"/>
-      <c r="C31" s="38"/>
-      <c r="D31" s="47"/>
-      <c r="E31" s="32"/>
+      <c r="B31" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C31" s="38">
+        <v>3</v>
+      </c>
+      <c r="D31" s="47" t="s">
+        <v>39</v>
+      </c>
+      <c r="E31" s="32">
+        <v>1.06E-2</v>
+      </c>
       <c r="F31" s="31">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>3.1800000000000002E-2</v>
       </c>
       <c r="G31" s="36"/>
       <c r="H31" s="43"/>
@@ -1540,13 +1663,21 @@
       <c r="A32" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="B32" s="6"/>
-      <c r="C32" s="38"/>
-      <c r="D32" s="47"/>
-      <c r="E32" s="32"/>
+      <c r="B32" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C32" s="38">
+        <v>3</v>
+      </c>
+      <c r="D32" s="47" t="s">
+        <v>41</v>
+      </c>
+      <c r="E32" s="32">
+        <v>0.02</v>
+      </c>
       <c r="F32" s="31">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.06</v>
       </c>
       <c r="G32" s="36"/>
       <c r="H32" s="43"/>
@@ -1688,13 +1819,13 @@
         <v>13</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C39" s="38">
         <v>2</v>
       </c>
       <c r="D39" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E39" s="32">
         <v>9.56</v>
@@ -1713,7 +1844,7 @@
       <c r="A40" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B40" s="59"/>
+      <c r="B40" s="58"/>
       <c r="C40" s="38"/>
       <c r="D40" s="47"/>
       <c r="E40" s="32"/>
@@ -1736,7 +1867,7 @@
       <c r="A41" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B41" s="59"/>
+      <c r="B41" s="58"/>
       <c r="C41" s="38"/>
       <c r="D41" s="47"/>
       <c r="E41" s="32"/>
@@ -2073,7 +2204,7 @@
       <c r="A57" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B57" s="60"/>
+      <c r="B57" s="59"/>
       <c r="C57" s="38"/>
       <c r="D57" s="47"/>
       <c r="E57" s="32"/>

</xml_diff>

<commit_message>
finalized component order form
</commit_message>
<xml_diff>
--- a/3_Hardware/9_Parts order form.xlsx
+++ b/3_Hardware/9_Parts order form.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bogda\Programming\PM4\PM4\3_Hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2139B156-0CFB-4712-B2D5-B353279DA633}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB444ABE-AF03-4F97-9AC2-18CBED4CC8D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="648" xr2:uid="{052C758A-BAC0-4DC7-8CE7-8521D951769E}"/>
   </bookViews>
@@ -16,16 +16,16 @@
     <sheet name="Sammel Bestellungen" sheetId="7" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Sammel Bestellungen'!$1:$4,'Sammel Bestellungen'!#REF!,'Sammel Bestellungen'!$15:$21,'Sammel Bestellungen'!#REF!</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Sammel Bestellungen'!$1:$4,'Sammel Bestellungen'!#REF!,'Sammel Bestellungen'!$7:$9,'Sammel Bestellungen'!#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <customWorkbookViews>
+    <customWorkbookView name="Mario Festini - Persönliche Ansicht" guid="{E7C05AF0-EEA1-11D3-A478-00D0B719A77E}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1276" windowHeight="888" tabRatio="454" activeSheetId="1"/>
+    <customWorkbookView name="Martin Studach - Persönliche Ansicht" guid="{41762A73-5BBF-11D4-A413-00D0B719978B}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1148" windowHeight="702" tabRatio="457" activeSheetId="1"/>
+    <customWorkbookView name="Werner Baumberger - Persönliche Ansicht" guid="{89927FE2-5BBA-11D4-87E4-00D0B719949C}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1276" windowHeight="908" tabRatio="457" activeSheetId="1" showStatusbar="0" showComments="commNone"/>
+    <customWorkbookView name="Patrick Mattioli - Persönliche Ansicht" guid="{D10A2CD0-5BB5-11D4-88A6-00D0B719D1AA}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1276" windowHeight="864" tabRatio="457" activeSheetId="1"/>
+    <customWorkbookView name="Patrik Jourdan - Persönliche Ansicht" guid="{ABF85D01-5BDF-11D4-A8DB-00D0B773D887}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1020" windowHeight="606" tabRatio="457" activeSheetId="1"/>
     <customWorkbookView name="mattioli - Persönliche Ansicht" guid="{6A967B41-C086-11D4-A516-00D0B719D1AA}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1276" windowHeight="890" activeSheetId="1"/>
-    <customWorkbookView name="Patrik Jourdan - Persönliche Ansicht" guid="{ABF85D01-5BDF-11D4-A8DB-00D0B773D887}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1020" windowHeight="606" tabRatio="457" activeSheetId="1"/>
-    <customWorkbookView name="Patrick Mattioli - Persönliche Ansicht" guid="{D10A2CD0-5BB5-11D4-88A6-00D0B719D1AA}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1276" windowHeight="864" tabRatio="457" activeSheetId="1"/>
-    <customWorkbookView name="Werner Baumberger - Persönliche Ansicht" guid="{89927FE2-5BBA-11D4-87E4-00D0B719949C}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1276" windowHeight="908" tabRatio="457" activeSheetId="1" showStatusbar="0" showComments="commNone"/>
-    <customWorkbookView name="Martin Studach - Persönliche Ansicht" guid="{41762A73-5BBF-11D4-A413-00D0B719978B}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1148" windowHeight="702" tabRatio="457" activeSheetId="1"/>
-    <customWorkbookView name="Mario Festini - Persönliche Ansicht" guid="{E7C05AF0-EEA1-11D3-A478-00D0B719A77E}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1276" windowHeight="888" tabRatio="454" activeSheetId="1"/>
   </customWorkbookViews>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="62">
   <si>
     <t>ArtNr.</t>
   </si>
@@ -76,9 +76,6 @@
     <t>Farnell</t>
   </si>
   <si>
-    <t>Distrelec</t>
-  </si>
-  <si>
     <t>spätester
 Bestell-termin</t>
   </si>
@@ -95,9 +92,6 @@
     <t>Achtung: Vor der Bestellung bitte unbedingt Lieferbarkeit prüfen. 
 - Art- Nr. ohne Leerzeichen eintragen. 
 - Mouser und Digikey nur wenn bei Distr./Farnell nicht erhätlich</t>
-  </si>
-  <si>
-    <t>Digikey</t>
   </si>
   <si>
     <t>Sammel- Bestellungen Dienstag Morgen
@@ -189,6 +183,72 @@
   <si>
     <t>Keramikvielschichtkondensator, SMD, 0.01 µF, 50 V, 0603 [Metrisch 1608], ± 10%, X7R</t>
   </si>
+  <si>
+    <t>CRG0603F10K</t>
+  </si>
+  <si>
+    <t>Chipwiderstand, Oberflächenmontage, 10 kohm, ± 1%, 100 mW, 0603 [Metrisch 1608]</t>
+  </si>
+  <si>
+    <t>CRCW06031M00FKEA</t>
+  </si>
+  <si>
+    <t>Chipwiderstand, Oberflächenmontage, 1 Mohm, ± 1%, 125 mW, 0603 [Metrisch 1608]</t>
+  </si>
+  <si>
+    <t>Chipwiderstand, Oberflächenmontage, 10 Mohm, ± 1%, 200 mW, 0603 [Metrisch 1608]</t>
+  </si>
+  <si>
+    <t>RCC060310M0FKEA</t>
+  </si>
+  <si>
+    <t>CRCW0603100KFKEA</t>
+  </si>
+  <si>
+    <t>Chipwiderstand, Oberflächenmontage, 100 kohm, ± 1%, 125 mW, 0603 [Metrisch 1608]</t>
+  </si>
+  <si>
+    <t>MCMR06X1001FTL</t>
+  </si>
+  <si>
+    <t>Chipwiderstand, Oberflächenmontage, Keramik, 1 kohm, ± 1%, 100 mW, 0603 [Metrisch 1608]</t>
+  </si>
+  <si>
+    <t>RC0603FR-07180KL</t>
+  </si>
+  <si>
+    <t>Chipwiderstand, Oberflächenmontage, 180 kohm, ± 1%, 100 mW, 0603 [Metrisch 1608]</t>
+  </si>
+  <si>
+    <t>RC0805FR-071KL</t>
+  </si>
+  <si>
+    <t>Chipwiderstand, Oberflächenmontage, 1 kohm, ± 1%, 125 mW, 0805 [Metrisch 2012]</t>
+  </si>
+  <si>
+    <t>CRCW0603360KFKEA</t>
+  </si>
+  <si>
+    <t>Chipwiderstand, Oberflächenmontage, 360 kohm, ± 1%, 125 mW, 0603 [Metrisch 1608]</t>
+  </si>
+  <si>
+    <t>RK73H1JTTD1404F</t>
+  </si>
+  <si>
+    <t>Chipwiderstand, Oberflächenmontage, 1.4 Mohm, ± 1%, 100 mW, 0603 [Metrisch 1608]</t>
+  </si>
+  <si>
+    <t>MCWR06X1102FTL</t>
+  </si>
+  <si>
+    <t>Chipwiderstand, Oberflächenmontage, 11 kohm, ± 1%, 100 mW, 0603 [Metrisch 1608]</t>
+  </si>
+  <si>
+    <t>MP008289</t>
+  </si>
+  <si>
+    <t>LED, Rot, Oberflächenmontage, 0603 [Metrisch: 1608], 20 mA, 2.4 V, 638 nm</t>
+  </si>
 </sst>
 </file>
 
@@ -199,7 +259,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.00_ ;[Red]\-#,##0.00\ "/>
     <numFmt numFmtId="166" formatCode="##\ ##\ ##"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="17">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -298,24 +358,7 @@
     </font>
     <font>
       <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
       <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF333333"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -355,9 +398,9 @@
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -427,9 +470,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -479,15 +519,9 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="16" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
       <protection locked="0"/>
@@ -496,52 +530,11 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="14" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
@@ -939,7 +932,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R1807"/>
+  <dimension ref="A1:R1756"/>
   <sheetFormatPr defaultColWidth="11.54296875" defaultRowHeight="12.5" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="15.26953125" style="2" bestFit="1" customWidth="1"/>
@@ -963,35 +956,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" customFormat="1" ht="60.75" customHeight="1">
-      <c r="A1" s="61" t="s">
-        <v>16</v>
-      </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="62" t="s">
+      <c r="A1" s="45" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="46" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
+      <c r="J1" s="46"/>
+      <c r="K1" s="46"/>
+      <c r="L1" s="46"/>
+      <c r="M1" s="46"/>
+      <c r="N1" s="46"/>
+      <c r="O1" s="46"/>
+      <c r="P1" s="46"/>
     </row>
     <row r="2" spans="1:16" customFormat="1" ht="3" customHeight="1">
-      <c r="A2" s="25"/>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="33"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="27"/>
+      <c r="A2" s="24"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="26"/>
       <c r="H2" s="6"/>
       <c r="I2" s="6"/>
       <c r="J2" s="7"/>
@@ -1020,13 +1013,13 @@
         <v>4</v>
       </c>
       <c r="G3" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="H3" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="I3" s="5" t="s">
         <v>11</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>12</v>
       </c>
       <c r="J3" s="5" t="s">
         <v>7</v>
@@ -1047,7 +1040,7 @@
       <c r="D4" s="12"/>
       <c r="E4" s="19"/>
       <c r="F4" s="20"/>
-      <c r="G4" s="28"/>
+      <c r="G4" s="27"/>
       <c r="H4" s="18"/>
       <c r="I4" s="14"/>
       <c r="J4" s="13"/>
@@ -1055,1856 +1048,967 @@
       <c r="L4" s="9"/>
       <c r="P4" s="14"/>
     </row>
-    <row r="5" spans="1:16" ht="21.75" customHeight="1">
-      <c r="A5" s="60" t="s">
-        <v>21</v>
+    <row r="5" spans="1:16" ht="13">
+      <c r="A5" s="2" t="s">
+        <v>19</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" s="38">
+        <v>17</v>
+      </c>
+      <c r="C5" s="2">
         <v>1</v>
       </c>
-      <c r="D5" s="47" t="s">
-        <v>20</v>
-      </c>
-      <c r="E5" s="24">
+      <c r="D5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" s="31">
         <v>9</v>
       </c>
-      <c r="F5" s="31">
-        <f t="shared" ref="F5:F18" si="0">C5*E5</f>
+      <c r="F5" s="30">
+        <f t="shared" ref="F5" si="0">C5*E5</f>
         <v>9</v>
       </c>
-      <c r="G5" s="36"/>
-      <c r="H5" s="39"/>
-      <c r="I5" s="39"/>
-      <c r="J5" s="37"/>
+      <c r="G5" s="35"/>
+      <c r="H5" s="38"/>
+      <c r="I5" s="38"/>
+      <c r="J5" s="36"/>
       <c r="K5" s="9"/>
       <c r="L5" s="9"/>
-      <c r="P5" s="44"/>
-    </row>
-    <row r="6" spans="1:16" s="4" customFormat="1" ht="39">
-      <c r="A6" s="4" t="s">
+      <c r="P5" s="41"/>
+    </row>
+    <row r="6" spans="1:16" ht="13">
+      <c r="B6" s="6"/>
+      <c r="D6"/>
+      <c r="E6" s="31"/>
+      <c r="F6" s="30"/>
+      <c r="G6" s="35"/>
+      <c r="H6" s="38"/>
+      <c r="I6" s="38"/>
+      <c r="J6" s="36"/>
+      <c r="K6" s="9"/>
+      <c r="L6" s="9"/>
+      <c r="P6" s="41"/>
+    </row>
+    <row r="7" spans="1:16" ht="39">
+      <c r="A7" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B7" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C7" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D7" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E7" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F7" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="G6" s="15" t="s">
+      <c r="G7" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="H7" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="I7" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="I6" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="J6" s="5" t="s">
+      <c r="J7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="K6" s="22"/>
-      <c r="L6" s="22"/>
-      <c r="M6" s="22"/>
-      <c r="N6" s="22"/>
-      <c r="O6" s="22"/>
-      <c r="P6" s="23" t="s">
+      <c r="P7" s="23" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="4.5" customHeight="1">
-      <c r="A7" s="11"/>
-      <c r="B7" s="11"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="19"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="28"/>
-      <c r="H7" s="18"/>
-      <c r="I7" s="14"/>
-      <c r="J7" s="13"/>
-      <c r="K7" s="9"/>
-      <c r="L7" s="9"/>
-      <c r="P7" s="14"/>
-    </row>
-    <row r="8" spans="1:16" ht="13">
-      <c r="A8" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F8" s="31">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G8" s="36"/>
-      <c r="H8" s="39"/>
-      <c r="I8" s="39"/>
-      <c r="K8" s="9"/>
-      <c r="L8" s="9"/>
-      <c r="P8" s="34"/>
-    </row>
-    <row r="9" spans="1:16" ht="13">
-      <c r="A9" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" s="57"/>
-      <c r="D9" s="48"/>
-      <c r="E9" s="24"/>
-      <c r="F9" s="31">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G9" s="36"/>
-      <c r="H9" s="39"/>
-      <c r="I9" s="39"/>
-      <c r="J9" s="37"/>
-      <c r="K9" s="9"/>
-      <c r="L9" s="9"/>
-      <c r="P9" s="45"/>
-    </row>
-    <row r="10" spans="1:16" ht="13">
-      <c r="A10" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" s="57"/>
-      <c r="D10" s="48"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="31">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G10" s="36"/>
-      <c r="H10" s="39"/>
-      <c r="I10" s="39"/>
-      <c r="J10" s="37"/>
-      <c r="K10" s="9"/>
-      <c r="L10" s="9"/>
-      <c r="P10" s="45"/>
-    </row>
-    <row r="11" spans="1:16" ht="13">
-      <c r="A11" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" s="57"/>
-      <c r="D11" s="48"/>
-      <c r="E11" s="24"/>
-      <c r="F11" s="52">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G11" s="36"/>
-      <c r="H11" s="39"/>
-      <c r="I11" s="39"/>
-      <c r="J11" s="37"/>
-      <c r="K11" s="9"/>
-      <c r="L11" s="9"/>
-      <c r="P11" s="45"/>
-    </row>
-    <row r="12" spans="1:16" ht="13">
-      <c r="A12" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B12" s="57"/>
-      <c r="C12" s="38"/>
-      <c r="D12" s="48"/>
-      <c r="E12" s="24"/>
-      <c r="F12" s="31">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G12" s="36"/>
-      <c r="H12" s="39"/>
-      <c r="I12" s="39"/>
-      <c r="J12" s="37"/>
-      <c r="K12" s="9"/>
-      <c r="L12" s="9"/>
-      <c r="P12" s="34"/>
+    <row r="8" spans="1:16" s="4" customFormat="1" ht="10">
+      <c r="A8" s="22"/>
+      <c r="B8" s="22"/>
+      <c r="C8" s="22"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="22"/>
+    </row>
+    <row r="9" spans="1:16" ht="6" customHeight="1">
+      <c r="A9" s="11"/>
+      <c r="B9" s="18"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="12"/>
+      <c r="E9" s="19"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="27"/>
+      <c r="H9" s="18"/>
+      <c r="I9" s="14"/>
+      <c r="J9" s="34"/>
+      <c r="P9" s="14"/>
+    </row>
+    <row r="10" spans="1:16" s="28" customFormat="1" ht="13">
+      <c r="A10" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" s="6">
+        <v>4029748</v>
+      </c>
+      <c r="C10" s="37">
+        <v>4</v>
+      </c>
+      <c r="D10" t="s">
+        <v>31</v>
+      </c>
+      <c r="E10" s="6">
+        <v>5.95</v>
+      </c>
+      <c r="F10" s="30">
+        <f t="shared" ref="F10:F31" si="1">C10*E10</f>
+        <v>23.8</v>
+      </c>
+      <c r="G10" s="35"/>
+      <c r="H10" s="38"/>
+      <c r="I10" s="38"/>
+      <c r="J10" s="36"/>
+      <c r="P10" s="41"/>
+    </row>
+    <row r="11" spans="1:16" s="28" customFormat="1" ht="13">
+      <c r="A11" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" s="37">
+        <v>22</v>
+      </c>
+      <c r="D11" t="s">
+        <v>21</v>
+      </c>
+      <c r="E11" s="31">
+        <v>3.9100000000000003E-2</v>
+      </c>
+      <c r="F11" s="30">
+        <f t="shared" si="1"/>
+        <v>0.86020000000000008</v>
+      </c>
+      <c r="G11" s="35"/>
+      <c r="H11" s="38"/>
+      <c r="I11" s="38"/>
+      <c r="J11" s="36"/>
+      <c r="P11" s="42"/>
+    </row>
+    <row r="12" spans="1:16" s="28" customFormat="1" ht="13">
+      <c r="A12" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" s="37">
+        <v>19</v>
+      </c>
+      <c r="D12" t="s">
+        <v>23</v>
+      </c>
+      <c r="E12" s="31">
+        <v>8.8300000000000003E-2</v>
+      </c>
+      <c r="F12" s="30">
+        <f t="shared" si="1"/>
+        <v>1.6777</v>
+      </c>
+      <c r="G12" s="35"/>
+      <c r="H12" s="38"/>
+      <c r="I12" s="38"/>
+      <c r="J12" s="36"/>
+      <c r="P12" s="33"/>
     </row>
     <row r="13" spans="1:16" ht="13">
-      <c r="A13" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B13" s="57"/>
-      <c r="D13" s="48"/>
-      <c r="E13" s="24"/>
-      <c r="F13" s="31">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G13" s="36"/>
-      <c r="H13" s="39"/>
-      <c r="I13" s="39"/>
-      <c r="J13" s="37"/>
-      <c r="K13" s="9"/>
-      <c r="L13" s="9"/>
-      <c r="P13" s="45"/>
-    </row>
-    <row r="14" spans="1:16" ht="13">
-      <c r="A14" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B14" s="57"/>
-      <c r="D14"/>
-      <c r="E14" s="24"/>
-      <c r="F14" s="31">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G14" s="36"/>
-      <c r="H14" s="39"/>
+      <c r="A13" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" s="2">
+        <v>13</v>
+      </c>
+      <c r="D13" t="s">
+        <v>33</v>
+      </c>
+      <c r="E13" s="31">
+        <v>0.224</v>
+      </c>
+      <c r="F13" s="30">
+        <f t="shared" si="1"/>
+        <v>2.9119999999999999</v>
+      </c>
+      <c r="G13" s="35"/>
+      <c r="H13" s="38"/>
+      <c r="I13" s="38"/>
+      <c r="J13" s="36"/>
+      <c r="P13" s="42"/>
+    </row>
+    <row r="14" spans="1:16" s="28" customFormat="1" ht="13">
+      <c r="A14" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" s="37">
+        <v>13</v>
+      </c>
+      <c r="D14" t="s">
+        <v>25</v>
+      </c>
+      <c r="E14" s="31">
+        <v>0.10100000000000001</v>
+      </c>
+      <c r="F14" s="30">
+        <f t="shared" si="1"/>
+        <v>1.3130000000000002</v>
+      </c>
+      <c r="G14" s="35"/>
+      <c r="H14" s="44"/>
       <c r="I14" s="39"/>
-      <c r="J14" s="37"/>
-      <c r="K14" s="9"/>
-      <c r="L14" s="9"/>
-      <c r="P14" s="45"/>
-    </row>
-    <row r="15" spans="1:16" ht="13">
-      <c r="A15" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B15" s="57"/>
-      <c r="D15"/>
-      <c r="E15" s="24"/>
-      <c r="F15" s="31">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G15" s="36"/>
+      <c r="J14" s="36"/>
+      <c r="P14" s="42"/>
+    </row>
+    <row r="15" spans="1:16" s="28" customFormat="1" ht="13">
+      <c r="A15" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" s="37">
+        <v>7</v>
+      </c>
+      <c r="D15" t="s">
+        <v>27</v>
+      </c>
+      <c r="E15" s="31">
+        <v>9.4E-2</v>
+      </c>
+      <c r="F15" s="30">
+        <f t="shared" si="1"/>
+        <v>0.65800000000000003</v>
+      </c>
+      <c r="G15" s="35"/>
       <c r="H15" s="39"/>
       <c r="I15" s="39"/>
-      <c r="J15" s="37"/>
-      <c r="K15" s="9"/>
-      <c r="L15" s="9"/>
-      <c r="P15" s="45"/>
-    </row>
-    <row r="16" spans="1:16" ht="13.5" customHeight="1">
-      <c r="A16" s="2" t="s">
+      <c r="J15" s="36"/>
+      <c r="P15" s="33"/>
+    </row>
+    <row r="16" spans="1:16" s="28" customFormat="1" ht="13">
+      <c r="A16" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" s="37">
+        <v>7</v>
+      </c>
+      <c r="D16" t="s">
+        <v>28</v>
+      </c>
+      <c r="E16" s="31">
+        <v>1.35E-2</v>
+      </c>
+      <c r="F16" s="30">
+        <f t="shared" si="1"/>
+        <v>9.4500000000000001E-2</v>
+      </c>
+      <c r="G16" s="35"/>
+      <c r="H16" s="38"/>
+      <c r="I16" s="39"/>
+      <c r="J16" s="36"/>
+      <c r="P16" s="41"/>
+    </row>
+    <row r="17" spans="1:16" ht="13">
+      <c r="A17" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="B17" s="6">
+        <v>885012206023</v>
+      </c>
+      <c r="C17" s="2">
+        <v>7</v>
+      </c>
+      <c r="D17" t="s">
+        <v>30</v>
+      </c>
+      <c r="E17" s="31">
+        <v>6.2300000000000001E-2</v>
+      </c>
+      <c r="F17" s="30">
+        <f t="shared" si="1"/>
+        <v>0.43609999999999999</v>
+      </c>
+      <c r="G17" s="35"/>
+      <c r="H17" s="40"/>
+      <c r="I17" s="39"/>
+      <c r="J17" s="36"/>
+      <c r="P17" s="42"/>
+    </row>
+    <row r="18" spans="1:16" s="28" customFormat="1" ht="13">
+      <c r="A18" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C18" s="37">
+        <v>4</v>
+      </c>
+      <c r="D18" s="43" t="s">
+        <v>35</v>
+      </c>
+      <c r="E18" s="31">
+        <v>0.14099999999999999</v>
+      </c>
+      <c r="F18" s="30">
+        <f t="shared" si="1"/>
+        <v>0.56399999999999995</v>
+      </c>
+      <c r="G18" s="35"/>
+      <c r="H18" s="40"/>
+      <c r="I18" s="39"/>
+      <c r="J18" s="36"/>
+      <c r="P18" s="41"/>
+    </row>
+    <row r="19" spans="1:16" s="28" customFormat="1" ht="13">
+      <c r="A19" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C19" s="37">
+        <v>4</v>
+      </c>
+      <c r="D19" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="E19" s="31">
+        <v>1.06E-2</v>
+      </c>
+      <c r="F19" s="30">
+        <f t="shared" si="1"/>
+        <v>4.24E-2</v>
+      </c>
+      <c r="G19" s="35"/>
+      <c r="H19" s="40"/>
+      <c r="I19" s="39"/>
+      <c r="J19" s="36"/>
+      <c r="P19" s="42"/>
+    </row>
+    <row r="20" spans="1:16" s="28" customFormat="1" ht="13">
+      <c r="A20" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C20" s="37">
+        <v>4</v>
+      </c>
+      <c r="D20" s="43" t="s">
+        <v>39</v>
+      </c>
+      <c r="E20" s="31">
+        <v>0.02</v>
+      </c>
+      <c r="F20" s="30">
+        <f t="shared" si="1"/>
+        <v>0.08</v>
+      </c>
+      <c r="G20" s="35"/>
+      <c r="H20" s="40"/>
+      <c r="I20" s="39"/>
+      <c r="J20" s="36"/>
+      <c r="P20" s="33"/>
+    </row>
+    <row r="21" spans="1:16" s="28" customFormat="1" ht="13">
+      <c r="A21" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C21" s="37">
+        <v>28</v>
+      </c>
+      <c r="D21" s="43" t="s">
+        <v>41</v>
+      </c>
+      <c r="E21" s="31">
+        <v>1.1900000000000001E-2</v>
+      </c>
+      <c r="F21" s="30">
+        <f t="shared" si="1"/>
+        <v>0.33320000000000005</v>
+      </c>
+      <c r="G21" s="35"/>
+      <c r="H21" s="40"/>
+      <c r="I21" s="39"/>
+      <c r="J21" s="36"/>
+      <c r="P21" s="41"/>
+    </row>
+    <row r="22" spans="1:16" s="28" customFormat="1" ht="13">
+      <c r="A22" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C22" s="2">
+        <v>28</v>
+      </c>
+      <c r="D22" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="E22" s="31">
+        <v>1.5299999999999999E-2</v>
+      </c>
+      <c r="F22" s="30">
+        <f t="shared" ref="F22:F30" si="2">C22*E22</f>
+        <v>0.4284</v>
+      </c>
+      <c r="G22" s="35"/>
+      <c r="H22" s="40"/>
+      <c r="I22" s="39"/>
+      <c r="J22" s="36"/>
+      <c r="P22" s="41"/>
+    </row>
+    <row r="23" spans="1:16" s="28" customFormat="1" ht="13">
+      <c r="A23" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C23" s="2">
+        <v>19</v>
+      </c>
+      <c r="D23" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="E23" s="31">
+        <v>3.3000000000000002E-2</v>
+      </c>
+      <c r="F23" s="30">
+        <f t="shared" si="2"/>
+        <v>0.627</v>
+      </c>
+      <c r="G23" s="35"/>
+      <c r="H23" s="40"/>
+      <c r="I23" s="39"/>
+      <c r="J23" s="36"/>
+      <c r="P23" s="41"/>
+    </row>
+    <row r="24" spans="1:16" s="28" customFormat="1" ht="13">
+      <c r="A24" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C24" s="2">
+        <v>13</v>
+      </c>
+      <c r="D24" s="43" t="s">
+        <v>47</v>
+      </c>
+      <c r="E24" s="31">
+        <v>1.5100000000000001E-2</v>
+      </c>
+      <c r="F24" s="30">
+        <f t="shared" si="2"/>
+        <v>0.1963</v>
+      </c>
+      <c r="G24" s="35"/>
+      <c r="H24" s="40"/>
+      <c r="I24" s="39"/>
+      <c r="J24" s="36"/>
+      <c r="P24" s="41"/>
+    </row>
+    <row r="25" spans="1:16" s="28" customFormat="1" ht="13">
+      <c r="A25" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C25" s="2">
+        <v>13</v>
+      </c>
+      <c r="D25" s="43" t="s">
+        <v>49</v>
+      </c>
+      <c r="E25" s="31">
+        <v>1.2E-2</v>
+      </c>
+      <c r="F25" s="30">
+        <f t="shared" si="2"/>
+        <v>0.156</v>
+      </c>
+      <c r="G25" s="35"/>
+      <c r="H25" s="40"/>
+      <c r="I25" s="39"/>
+      <c r="J25" s="36"/>
+      <c r="P25" s="41"/>
+    </row>
+    <row r="26" spans="1:16" s="28" customFormat="1" ht="13">
+      <c r="A26" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C26" s="2">
+        <v>7</v>
+      </c>
+      <c r="D26" s="43" t="s">
+        <v>51</v>
+      </c>
+      <c r="E26" s="31">
+        <v>6.8999999999999999E-3</v>
+      </c>
+      <c r="F26" s="30">
+        <f t="shared" si="2"/>
+        <v>4.8299999999999996E-2</v>
+      </c>
+      <c r="G26" s="35"/>
+      <c r="H26" s="40"/>
+      <c r="I26" s="39"/>
+      <c r="J26" s="36"/>
+      <c r="P26" s="41"/>
+    </row>
+    <row r="27" spans="1:16" s="28" customFormat="1" ht="13">
+      <c r="A27" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C27" s="2">
+        <v>4</v>
+      </c>
+      <c r="D27" s="43" t="s">
+        <v>53</v>
+      </c>
+      <c r="E27" s="31">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="F27" s="30">
+        <f t="shared" si="2"/>
+        <v>2.8000000000000001E-2</v>
+      </c>
+      <c r="G27" s="35"/>
+      <c r="H27" s="40"/>
+      <c r="I27" s="39"/>
+      <c r="J27" s="36"/>
+      <c r="P27" s="41"/>
+    </row>
+    <row r="28" spans="1:16" s="28" customFormat="1" ht="13">
+      <c r="A28" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="C28" s="2">
+        <v>4</v>
+      </c>
+      <c r="D28" s="43" t="s">
+        <v>55</v>
+      </c>
+      <c r="E28" s="31">
+        <v>1.9199999999999998E-2</v>
+      </c>
+      <c r="F28" s="30">
+        <f t="shared" si="2"/>
+        <v>7.6799999999999993E-2</v>
+      </c>
+      <c r="G28" s="35"/>
+      <c r="H28" s="40"/>
+      <c r="I28" s="39"/>
+      <c r="J28" s="36"/>
+      <c r="P28" s="41"/>
+    </row>
+    <row r="29" spans="1:16" s="28" customFormat="1" ht="13">
+      <c r="A29" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C29" s="2">
+        <v>4</v>
+      </c>
+      <c r="D29" s="43" t="s">
+        <v>57</v>
+      </c>
+      <c r="E29" s="31">
+        <v>1.4200000000000001E-2</v>
+      </c>
+      <c r="F29" s="30">
+        <f t="shared" si="2"/>
+        <v>5.6800000000000003E-2</v>
+      </c>
+      <c r="G29" s="35"/>
+      <c r="H29" s="40"/>
+      <c r="I29" s="39"/>
+      <c r="J29" s="36"/>
+      <c r="P29" s="41"/>
+    </row>
+    <row r="30" spans="1:16" s="28" customFormat="1" ht="13">
+      <c r="A30" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="C30" s="2">
+        <v>4</v>
+      </c>
+      <c r="D30" s="43" t="s">
+        <v>59</v>
+      </c>
+      <c r="E30" s="31">
+        <v>4.5999999999999999E-3</v>
+      </c>
+      <c r="F30" s="30">
+        <f t="shared" si="2"/>
+        <v>1.84E-2</v>
+      </c>
+      <c r="G30" s="35"/>
+      <c r="H30" s="40"/>
+      <c r="I30" s="39"/>
+      <c r="J30" s="36"/>
+      <c r="P30" s="41"/>
+    </row>
+    <row r="31" spans="1:16" ht="13">
+      <c r="A31" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C31" s="2">
+        <v>7</v>
+      </c>
+      <c r="D31" s="43" t="s">
+        <v>61</v>
+      </c>
+      <c r="E31" s="31">
+        <v>0.13600000000000001</v>
+      </c>
+      <c r="F31" s="30">
+        <f t="shared" si="1"/>
+        <v>0.95200000000000007</v>
+      </c>
+      <c r="G31" s="35"/>
+      <c r="H31" s="40"/>
+      <c r="I31" s="39"/>
+      <c r="J31" s="36"/>
+      <c r="P31" s="42"/>
+    </row>
+    <row r="32" spans="1:16" s="28" customFormat="1" ht="13">
+      <c r="A32" s="29"/>
+      <c r="B32" s="6"/>
+      <c r="C32" s="37"/>
+      <c r="D32" s="43"/>
+      <c r="E32" s="31"/>
+      <c r="F32" s="30"/>
+      <c r="G32" s="35"/>
+      <c r="H32" s="40"/>
+      <c r="I32" s="39"/>
+      <c r="J32" s="36"/>
+      <c r="P32" s="41"/>
+    </row>
+    <row r="33" spans="1:16" s="28" customFormat="1" ht="39">
+      <c r="A33" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B33" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="C33" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="D33" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="E33" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="F33" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="G33" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="B16" s="57"/>
-      <c r="D16"/>
-      <c r="E16" s="24"/>
-      <c r="F16" s="31">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G16" s="36"/>
-      <c r="H16" s="39"/>
-      <c r="I16" s="40"/>
-      <c r="J16" s="37"/>
-      <c r="K16" s="9"/>
-      <c r="L16" s="9"/>
-      <c r="P16" s="45"/>
-    </row>
-    <row r="17" spans="1:16" ht="13">
-      <c r="A17" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B17" s="57"/>
-      <c r="D17"/>
-      <c r="E17" s="24"/>
-      <c r="F17" s="31">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G17" s="36"/>
-      <c r="H17" s="39"/>
-      <c r="I17" s="40"/>
-      <c r="J17" s="37"/>
-      <c r="K17" s="9"/>
-      <c r="L17" s="9"/>
-      <c r="P17" s="45"/>
-    </row>
-    <row r="18" spans="1:16" ht="13">
-      <c r="A18" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B18" s="57"/>
-      <c r="D18"/>
-      <c r="E18" s="24"/>
-      <c r="F18" s="31">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G18" s="36"/>
-      <c r="H18" s="39"/>
-      <c r="I18" s="40"/>
-      <c r="J18" s="37"/>
-      <c r="K18" s="9"/>
-      <c r="L18" s="9"/>
-      <c r="P18" s="45"/>
-    </row>
-    <row r="19" spans="1:16" ht="39">
-      <c r="A19" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B19" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="C19" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="D19" s="10" t="s">
+      <c r="H33" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I33" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="J33" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K33" s="1"/>
+      <c r="L33" s="1"/>
+      <c r="M33" s="1"/>
+      <c r="N33" s="1"/>
+      <c r="O33" s="1"/>
+      <c r="P33" s="23" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" s="28" customFormat="1">
+      <c r="A34" s="22"/>
+      <c r="B34" s="22"/>
+      <c r="C34" s="22"/>
+      <c r="D34" s="22"/>
+      <c r="E34" s="22"/>
+      <c r="F34" s="4"/>
+      <c r="G34" s="4"/>
+      <c r="H34" s="4"/>
+      <c r="I34" s="4"/>
+      <c r="J34" s="4"/>
+      <c r="K34" s="4"/>
+      <c r="L34" s="4"/>
+      <c r="M34" s="4"/>
+      <c r="N34" s="4"/>
+      <c r="O34" s="4"/>
+      <c r="P34" s="4"/>
+    </row>
+    <row r="35" spans="1:16" s="28" customFormat="1" ht="13">
+      <c r="A35" s="11"/>
+      <c r="B35" s="18"/>
+      <c r="C35" s="11"/>
+      <c r="D35" s="12"/>
+      <c r="E35" s="19"/>
+      <c r="F35" s="8"/>
+      <c r="G35" s="27"/>
+      <c r="H35" s="18"/>
+      <c r="I35" s="14"/>
+      <c r="J35" s="34"/>
+      <c r="K35" s="1"/>
+      <c r="L35" s="1"/>
+      <c r="M35" s="1"/>
+      <c r="N35" s="1"/>
+      <c r="O35" s="1"/>
+      <c r="P35" s="14"/>
+    </row>
+    <row r="36" spans="1:16" s="28" customFormat="1" ht="13">
+      <c r="A36" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C36" s="37">
         <v>2</v>
       </c>
-      <c r="E19" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="F19" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="G19" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="H19" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="I19" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="J19" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="P19" s="23" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="20" spans="1:16" s="4" customFormat="1" ht="10">
-      <c r="A20" s="22"/>
-      <c r="B20" s="22"/>
-      <c r="C20" s="22"/>
-      <c r="D20" s="22"/>
-      <c r="E20" s="22"/>
-    </row>
-    <row r="21" spans="1:16" ht="6" customHeight="1">
-      <c r="A21" s="11"/>
-      <c r="B21" s="18"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="12"/>
-      <c r="E21" s="19"/>
-      <c r="F21" s="8"/>
-      <c r="G21" s="28"/>
-      <c r="H21" s="18"/>
-      <c r="I21" s="14"/>
-      <c r="J21" s="35"/>
-      <c r="P21" s="14"/>
-    </row>
-    <row r="22" spans="1:16" s="29" customFormat="1" ht="13">
-      <c r="A22" s="30" t="s">
-        <v>8</v>
-      </c>
-      <c r="B22" s="6">
-        <v>4029748</v>
-      </c>
-      <c r="C22" s="38">
-        <v>4</v>
-      </c>
-      <c r="D22" t="s">
-        <v>33</v>
-      </c>
-      <c r="E22" s="6">
-        <v>5.95</v>
-      </c>
-      <c r="F22" s="31">
-        <f t="shared" ref="F22:F34" si="1">C22*E22</f>
-        <v>23.8</v>
-      </c>
-      <c r="G22" s="36"/>
-      <c r="H22" s="39"/>
-      <c r="I22" s="39"/>
-      <c r="J22" s="37"/>
-      <c r="P22" s="44"/>
-    </row>
-    <row r="23" spans="1:16" s="29" customFormat="1" ht="13">
-      <c r="A23" s="30" t="s">
-        <v>8</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C23" s="38">
-        <v>21</v>
-      </c>
-      <c r="D23" t="s">
-        <v>23</v>
-      </c>
-      <c r="E23" s="32">
-        <v>3.9100000000000003E-2</v>
-      </c>
-      <c r="F23" s="31">
-        <f t="shared" si="1"/>
-        <v>0.82110000000000005</v>
-      </c>
-      <c r="G23" s="36"/>
-      <c r="H23" s="39"/>
-      <c r="I23" s="39"/>
-      <c r="J23" s="37"/>
-      <c r="P23" s="46"/>
-    </row>
-    <row r="24" spans="1:16" s="29" customFormat="1" ht="13">
-      <c r="A24" s="30" t="s">
-        <v>8</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C24" s="38">
-        <v>18</v>
-      </c>
-      <c r="D24" t="s">
-        <v>25</v>
-      </c>
-      <c r="E24" s="32">
-        <v>8.8300000000000003E-2</v>
-      </c>
-      <c r="F24" s="31">
-        <f t="shared" si="1"/>
-        <v>1.5894000000000001</v>
-      </c>
-      <c r="G24" s="36"/>
-      <c r="H24" s="39"/>
-      <c r="I24" s="39"/>
-      <c r="J24" s="37"/>
-      <c r="P24" s="34"/>
-    </row>
-    <row r="25" spans="1:16" ht="13">
-      <c r="A25" s="30" t="s">
-        <v>8</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="C25" s="2">
-        <v>12</v>
-      </c>
-      <c r="D25" t="s">
-        <v>35</v>
-      </c>
-      <c r="E25" s="32">
-        <v>0.224</v>
-      </c>
-      <c r="F25" s="31">
-        <f t="shared" si="1"/>
-        <v>2.6880000000000002</v>
-      </c>
-      <c r="G25" s="36"/>
-      <c r="H25" s="39"/>
-      <c r="I25" s="39"/>
-      <c r="J25" s="37"/>
-      <c r="P25" s="46"/>
-    </row>
-    <row r="26" spans="1:16" s="29" customFormat="1" ht="13">
-      <c r="A26" s="30" t="s">
-        <v>8</v>
-      </c>
-      <c r="B26" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C26" s="38">
-        <v>12</v>
-      </c>
-      <c r="D26" t="s">
-        <v>27</v>
-      </c>
-      <c r="E26" s="32">
-        <v>0.10100000000000001</v>
-      </c>
-      <c r="F26" s="31">
-        <f t="shared" si="1"/>
-        <v>1.2120000000000002</v>
-      </c>
-      <c r="G26" s="36"/>
-      <c r="H26" s="51"/>
-      <c r="I26" s="41"/>
-      <c r="J26" s="37"/>
-      <c r="P26" s="46"/>
-    </row>
-    <row r="27" spans="1:16" s="29" customFormat="1" ht="13">
-      <c r="A27" s="30" t="s">
-        <v>8</v>
-      </c>
-      <c r="B27" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C27" s="38">
-        <v>6</v>
-      </c>
-      <c r="D27" t="s">
-        <v>29</v>
-      </c>
-      <c r="E27" s="32">
-        <v>9.4E-2</v>
-      </c>
-      <c r="F27" s="31">
-        <f t="shared" si="1"/>
-        <v>0.56400000000000006</v>
-      </c>
-      <c r="G27" s="36"/>
-      <c r="H27" s="41"/>
-      <c r="I27" s="41"/>
-      <c r="J27" s="37"/>
-      <c r="P27" s="34"/>
-    </row>
-    <row r="28" spans="1:16" s="29" customFormat="1" ht="13">
-      <c r="A28" s="30" t="s">
-        <v>8</v>
-      </c>
-      <c r="B28" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C28" s="38">
-        <v>6</v>
-      </c>
-      <c r="D28" t="s">
-        <v>30</v>
-      </c>
-      <c r="E28" s="32">
-        <v>1.35E-2</v>
-      </c>
-      <c r="F28" s="31">
-        <f t="shared" si="1"/>
-        <v>8.1000000000000003E-2</v>
-      </c>
-      <c r="G28" s="36"/>
-      <c r="H28" s="39"/>
-      <c r="I28" s="41"/>
-      <c r="J28" s="37"/>
-      <c r="P28" s="44"/>
-    </row>
-    <row r="29" spans="1:16" ht="13">
-      <c r="A29" s="30" t="s">
-        <v>8</v>
-      </c>
-      <c r="B29" s="6">
-        <v>885012206023</v>
-      </c>
-      <c r="C29" s="2">
-        <v>6</v>
-      </c>
-      <c r="D29" t="s">
-        <v>32</v>
-      </c>
-      <c r="E29" s="32">
-        <v>6.2300000000000001E-2</v>
-      </c>
-      <c r="F29" s="31">
-        <f t="shared" si="1"/>
-        <v>0.37380000000000002</v>
-      </c>
-      <c r="G29" s="36"/>
-      <c r="H29" s="43"/>
-      <c r="I29" s="41"/>
-      <c r="J29" s="37"/>
-      <c r="P29" s="46"/>
-    </row>
-    <row r="30" spans="1:16" s="29" customFormat="1" ht="13">
-      <c r="A30" s="30" t="s">
-        <v>8</v>
-      </c>
-      <c r="B30" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C30" s="38">
-        <v>3</v>
-      </c>
-      <c r="D30" s="47" t="s">
-        <v>37</v>
-      </c>
-      <c r="E30" s="32">
-        <v>0.14099999999999999</v>
-      </c>
-      <c r="F30" s="31">
-        <f t="shared" si="1"/>
-        <v>0.42299999999999993</v>
-      </c>
-      <c r="G30" s="36"/>
-      <c r="H30" s="43"/>
-      <c r="I30" s="41"/>
-      <c r="J30" s="37"/>
-      <c r="P30" s="44"/>
-    </row>
-    <row r="31" spans="1:16" s="29" customFormat="1" ht="13">
-      <c r="A31" s="30" t="s">
-        <v>8</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C31" s="38">
-        <v>3</v>
-      </c>
-      <c r="D31" s="47" t="s">
-        <v>39</v>
-      </c>
-      <c r="E31" s="32">
-        <v>1.06E-2</v>
-      </c>
-      <c r="F31" s="31">
-        <f t="shared" si="1"/>
-        <v>3.1800000000000002E-2</v>
-      </c>
-      <c r="G31" s="36"/>
-      <c r="H31" s="43"/>
-      <c r="I31" s="41"/>
-      <c r="J31" s="37"/>
-      <c r="P31" s="46"/>
-    </row>
-    <row r="32" spans="1:16" s="29" customFormat="1" ht="13">
-      <c r="A32" s="30" t="s">
-        <v>8</v>
-      </c>
-      <c r="B32" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C32" s="38">
-        <v>3</v>
-      </c>
-      <c r="D32" s="47" t="s">
-        <v>41</v>
-      </c>
-      <c r="E32" s="32">
-        <v>0.02</v>
-      </c>
-      <c r="F32" s="31">
-        <f t="shared" si="1"/>
-        <v>0.06</v>
-      </c>
-      <c r="G32" s="36"/>
-      <c r="H32" s="43"/>
-      <c r="I32" s="41"/>
-      <c r="J32" s="37"/>
-      <c r="P32" s="34"/>
-    </row>
-    <row r="33" spans="1:16" s="29" customFormat="1" ht="13">
-      <c r="A33" s="30" t="s">
-        <v>8</v>
-      </c>
-      <c r="B33" s="6"/>
-      <c r="C33" s="38"/>
-      <c r="D33" s="47"/>
-      <c r="E33" s="32"/>
-      <c r="F33" s="31">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G33" s="36"/>
-      <c r="H33" s="43"/>
-      <c r="I33" s="41"/>
-      <c r="J33" s="37"/>
-      <c r="P33" s="44"/>
-    </row>
-    <row r="34" spans="1:16" ht="13">
-      <c r="A34" s="30" t="s">
-        <v>8</v>
-      </c>
-      <c r="B34" s="6"/>
-      <c r="D34" s="47"/>
-      <c r="E34" s="32"/>
-      <c r="F34" s="31">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G34" s="36"/>
-      <c r="H34" s="43"/>
-      <c r="I34" s="41"/>
-      <c r="J34" s="37"/>
-      <c r="P34" s="46"/>
-    </row>
-    <row r="35" spans="1:16" s="29" customFormat="1" ht="13">
-      <c r="A35" s="30" t="s">
-        <v>8</v>
-      </c>
-      <c r="B35" s="6"/>
-      <c r="C35" s="38"/>
-      <c r="D35" s="47"/>
-      <c r="E35" s="32"/>
-      <c r="F35" s="31">
-        <f>C35*E35</f>
-        <v>0</v>
-      </c>
-      <c r="G35" s="36"/>
-      <c r="H35" s="43"/>
-      <c r="I35" s="41"/>
-      <c r="J35" s="37"/>
-      <c r="P35" s="44"/>
-    </row>
-    <row r="36" spans="1:16" s="29" customFormat="1" ht="39">
-      <c r="A36" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B36" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="C36" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="D36" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="E36" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="F36" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="G36" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="H36" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="I36" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="J36" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="K36" s="1"/>
-      <c r="L36" s="1"/>
-      <c r="M36" s="1"/>
-      <c r="N36" s="1"/>
-      <c r="O36" s="1"/>
-      <c r="P36" s="23" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="37" spans="1:16" s="29" customFormat="1">
-      <c r="A37" s="22"/>
-      <c r="B37" s="22"/>
-      <c r="C37" s="22"/>
-      <c r="D37" s="22"/>
-      <c r="E37" s="22"/>
-      <c r="F37" s="4"/>
-      <c r="G37" s="4"/>
-      <c r="H37" s="4"/>
-      <c r="I37" s="4"/>
-      <c r="J37" s="4"/>
-      <c r="K37" s="4"/>
-      <c r="L37" s="4"/>
-      <c r="M37" s="4"/>
-      <c r="N37" s="4"/>
-      <c r="O37" s="4"/>
-      <c r="P37" s="4"/>
-    </row>
-    <row r="38" spans="1:16" s="29" customFormat="1" ht="13">
-      <c r="A38" s="11"/>
-      <c r="B38" s="18"/>
-      <c r="C38" s="11"/>
-      <c r="D38" s="12"/>
-      <c r="E38" s="19"/>
-      <c r="F38" s="8"/>
-      <c r="G38" s="28"/>
-      <c r="H38" s="18"/>
-      <c r="I38" s="14"/>
-      <c r="J38" s="35"/>
-      <c r="K38" s="1"/>
-      <c r="L38" s="1"/>
-      <c r="M38" s="1"/>
-      <c r="N38" s="1"/>
-      <c r="O38" s="1"/>
-      <c r="P38" s="14"/>
-    </row>
-    <row r="39" spans="1:16" s="29" customFormat="1" ht="13">
-      <c r="A39" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B39" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C39" s="38">
-        <v>2</v>
-      </c>
-      <c r="D39" t="s">
-        <v>17</v>
-      </c>
-      <c r="E39" s="32">
+      <c r="D36" t="s">
+        <v>15</v>
+      </c>
+      <c r="E36" s="31">
         <v>9.56</v>
       </c>
-      <c r="F39" s="31">
-        <f t="shared" ref="F39:F63" si="2">C39*E39</f>
+      <c r="F36" s="30">
+        <f t="shared" ref="F36" si="3">C36*E36</f>
         <v>19.12</v>
       </c>
-      <c r="G39" s="36"/>
-      <c r="H39" s="41"/>
-      <c r="I39" s="41"/>
-      <c r="J39" s="37"/>
-      <c r="P39" s="44"/>
-    </row>
-    <row r="40" spans="1:16" ht="13">
-      <c r="A40" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B40" s="58"/>
-      <c r="C40" s="38"/>
-      <c r="D40" s="47"/>
-      <c r="E40" s="32"/>
-      <c r="F40" s="31">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G40" s="36"/>
-      <c r="H40" s="41"/>
-      <c r="I40" s="41"/>
-      <c r="J40" s="37"/>
-      <c r="K40" s="29"/>
-      <c r="L40" s="29"/>
-      <c r="M40" s="29"/>
-      <c r="N40" s="29"/>
-      <c r="O40" s="29"/>
-      <c r="P40" s="46"/>
-    </row>
-    <row r="41" spans="1:16" s="29" customFormat="1" ht="13">
-      <c r="A41" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B41" s="58"/>
-      <c r="C41" s="38"/>
-      <c r="D41" s="47"/>
-      <c r="E41" s="32"/>
-      <c r="F41" s="31">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G41" s="36"/>
-      <c r="H41" s="41"/>
-      <c r="I41" s="42"/>
-      <c r="J41" s="37"/>
-      <c r="P41" s="34"/>
-    </row>
-    <row r="42" spans="1:16" s="29" customFormat="1" ht="13">
-      <c r="A42" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B42" s="6"/>
-      <c r="C42" s="38"/>
-      <c r="D42"/>
-      <c r="E42" s="32"/>
-      <c r="F42" s="31">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G42" s="36"/>
-      <c r="H42" s="51"/>
-      <c r="I42" s="41"/>
-      <c r="J42" s="37"/>
-      <c r="P42" s="44"/>
-    </row>
-    <row r="43" spans="1:16" s="29" customFormat="1" ht="13">
-      <c r="A43" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B43" s="6"/>
-      <c r="C43" s="2"/>
-      <c r="D43"/>
-      <c r="E43" s="32"/>
-      <c r="F43" s="31">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G43" s="36"/>
-      <c r="H43" s="51"/>
-      <c r="I43" s="41"/>
-      <c r="J43" s="37"/>
-      <c r="K43" s="1"/>
-      <c r="L43" s="1"/>
-      <c r="M43" s="1"/>
-      <c r="N43" s="1"/>
-      <c r="O43" s="1"/>
-      <c r="P43" s="46"/>
-    </row>
-    <row r="44" spans="1:16" ht="13">
-      <c r="A44" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B44" s="6"/>
-      <c r="C44" s="38"/>
-      <c r="D44"/>
-      <c r="E44" s="32"/>
-      <c r="F44" s="31">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G44" s="36"/>
-      <c r="H44" s="51"/>
-      <c r="I44" s="41"/>
-      <c r="J44" s="37"/>
-      <c r="K44" s="29"/>
-      <c r="L44" s="29"/>
-      <c r="M44" s="29"/>
-      <c r="N44" s="29"/>
-      <c r="O44" s="29"/>
-      <c r="P44" s="44"/>
-    </row>
-    <row r="45" spans="1:16" ht="13">
-      <c r="A45" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B45" s="6"/>
-      <c r="C45" s="38"/>
-      <c r="D45"/>
-      <c r="E45" s="32"/>
-      <c r="F45" s="31">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G45" s="36"/>
-      <c r="H45" s="51"/>
-      <c r="I45" s="41"/>
-      <c r="J45" s="37"/>
-      <c r="K45" s="29"/>
-      <c r="L45" s="29"/>
-      <c r="M45" s="29"/>
-      <c r="N45" s="29"/>
-      <c r="O45" s="29"/>
-      <c r="P45" s="46"/>
-    </row>
-    <row r="46" spans="1:16" ht="13">
-      <c r="A46" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B46" s="6"/>
-      <c r="C46" s="38"/>
-      <c r="D46"/>
-      <c r="E46" s="32"/>
-      <c r="F46" s="31">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G46" s="36"/>
-      <c r="H46" s="51"/>
-      <c r="I46" s="41"/>
-      <c r="J46" s="37"/>
-      <c r="K46" s="29"/>
-      <c r="L46" s="29"/>
-      <c r="M46" s="29"/>
-      <c r="N46" s="29"/>
-      <c r="O46" s="29"/>
-      <c r="P46" s="34"/>
-    </row>
-    <row r="47" spans="1:16" ht="13">
-      <c r="A47" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B47" s="6"/>
-      <c r="C47" s="38"/>
-      <c r="D47"/>
-      <c r="E47" s="32"/>
-      <c r="F47" s="31">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G47" s="36"/>
-      <c r="H47" s="51"/>
-      <c r="I47" s="41"/>
-      <c r="J47" s="37"/>
-      <c r="K47" s="29"/>
-      <c r="L47" s="29"/>
-      <c r="M47" s="29"/>
-      <c r="N47" s="29"/>
-      <c r="O47" s="29"/>
-      <c r="P47" s="44"/>
-    </row>
-    <row r="48" spans="1:16" ht="13">
-      <c r="A48" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B48" s="6"/>
-      <c r="D48"/>
-      <c r="E48" s="32"/>
-      <c r="F48" s="31">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G48" s="36"/>
-      <c r="H48" s="51"/>
-      <c r="I48" s="41"/>
-      <c r="J48" s="37"/>
-      <c r="P48" s="46"/>
-    </row>
-    <row r="49" spans="1:16" ht="13">
-      <c r="A49" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B49" s="6"/>
-      <c r="C49" s="38"/>
-      <c r="D49" s="50"/>
-      <c r="E49" s="32"/>
-      <c r="F49" s="31">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G49" s="36"/>
-      <c r="H49" s="51"/>
-      <c r="I49" s="41"/>
-      <c r="J49" s="37"/>
-      <c r="K49" s="29"/>
-      <c r="L49" s="29"/>
-      <c r="M49" s="29"/>
-      <c r="N49" s="29"/>
-      <c r="O49" s="29"/>
-      <c r="P49" s="44"/>
-    </row>
-    <row r="50" spans="1:16" s="54" customFormat="1" ht="13">
-      <c r="A50" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B50" s="6"/>
-      <c r="C50" s="53"/>
-      <c r="D50" s="50"/>
-      <c r="E50" s="6"/>
-      <c r="F50" s="52">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G50" s="36"/>
-      <c r="H50" s="41"/>
-      <c r="I50" s="41"/>
-      <c r="J50" s="37"/>
-      <c r="P50" s="44"/>
-    </row>
-    <row r="51" spans="1:16" ht="13">
-      <c r="A51" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B51" s="6"/>
-      <c r="C51" s="53"/>
-      <c r="D51" s="55"/>
-      <c r="E51" s="56"/>
-      <c r="F51" s="52">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G51" s="36"/>
-      <c r="H51" s="41"/>
-      <c r="I51" s="41"/>
-      <c r="J51" s="37"/>
-      <c r="K51" s="54"/>
-      <c r="L51" s="54"/>
-      <c r="M51" s="54"/>
-      <c r="N51" s="54"/>
-      <c r="O51" s="54"/>
-      <c r="P51" s="46"/>
-    </row>
-    <row r="52" spans="1:16" s="54" customFormat="1" ht="13">
-      <c r="A52" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B52" s="6"/>
-      <c r="C52" s="53"/>
-      <c r="D52" s="50"/>
-      <c r="E52" s="56"/>
-      <c r="F52" s="52">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G52" s="36"/>
-      <c r="H52" s="41"/>
-      <c r="I52" s="41"/>
-      <c r="J52" s="37"/>
-      <c r="P52" s="34"/>
-    </row>
-    <row r="53" spans="1:16" s="54" customFormat="1" ht="13">
-      <c r="A53" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B53" s="6"/>
-      <c r="C53" s="53"/>
-      <c r="D53" s="50"/>
-      <c r="E53" s="56"/>
-      <c r="F53" s="52">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G53" s="36"/>
-      <c r="H53" s="41"/>
-      <c r="I53" s="41"/>
-      <c r="J53" s="37"/>
-      <c r="P53" s="44"/>
-    </row>
-    <row r="54" spans="1:16" s="54" customFormat="1" ht="13">
-      <c r="A54" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B54" s="6"/>
-      <c r="C54" s="2"/>
-      <c r="D54" s="50"/>
-      <c r="E54" s="56"/>
-      <c r="F54" s="52">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G54" s="36"/>
-      <c r="H54" s="41"/>
-      <c r="I54" s="41"/>
-      <c r="J54" s="37"/>
-      <c r="K54" s="1"/>
-      <c r="L54" s="1"/>
-      <c r="M54" s="1"/>
-      <c r="N54" s="1"/>
-      <c r="O54" s="1"/>
-      <c r="P54" s="46"/>
-    </row>
-    <row r="55" spans="1:16" ht="13">
-      <c r="A55" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B55" s="6"/>
-      <c r="C55" s="53"/>
-      <c r="D55" s="50"/>
-      <c r="E55" s="56"/>
-      <c r="F55" s="52">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G55" s="36"/>
-      <c r="H55" s="41"/>
-      <c r="I55" s="41"/>
-      <c r="J55" s="37"/>
-      <c r="K55" s="54"/>
-      <c r="L55" s="54"/>
-      <c r="M55" s="54"/>
-      <c r="N55" s="54"/>
-      <c r="O55" s="54"/>
-      <c r="P55" s="44"/>
-    </row>
-    <row r="56" spans="1:16" ht="13">
-      <c r="A56" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B56" s="6"/>
-      <c r="C56" s="53"/>
-      <c r="D56" s="50"/>
-      <c r="E56" s="56"/>
-      <c r="F56" s="52">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G56" s="36"/>
-      <c r="H56" s="51"/>
-      <c r="I56" s="41"/>
-      <c r="J56" s="37"/>
-      <c r="K56" s="54"/>
-      <c r="L56" s="54"/>
-      <c r="M56" s="54"/>
-      <c r="N56" s="54"/>
-      <c r="O56" s="54"/>
-      <c r="P56" s="46"/>
-    </row>
-    <row r="57" spans="1:16" ht="13">
-      <c r="A57" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B57" s="59"/>
-      <c r="C57" s="38"/>
-      <c r="D57" s="47"/>
-      <c r="E57" s="32"/>
-      <c r="F57" s="31">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G57" s="36"/>
-      <c r="H57" s="51"/>
-      <c r="I57" s="41"/>
-      <c r="J57" s="37"/>
-      <c r="K57" s="29"/>
-      <c r="L57" s="29"/>
-      <c r="M57" s="29"/>
-      <c r="N57" s="29"/>
-      <c r="O57" s="29"/>
-      <c r="P57" s="46"/>
-    </row>
-    <row r="58" spans="1:16" ht="13">
-      <c r="A58" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B58" s="6"/>
-      <c r="C58" s="38"/>
-      <c r="D58" s="47"/>
-      <c r="E58" s="32"/>
-      <c r="F58" s="31">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G58" s="36"/>
-      <c r="H58" s="43"/>
-      <c r="I58" s="41"/>
-      <c r="J58" s="37"/>
-      <c r="K58" s="29"/>
-      <c r="L58" s="29"/>
-      <c r="M58" s="29"/>
-      <c r="N58" s="29"/>
-      <c r="O58" s="29"/>
-      <c r="P58" s="34"/>
-    </row>
-    <row r="59" spans="1:16" ht="13">
-      <c r="A59" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B59" s="6"/>
-      <c r="C59" s="38"/>
-      <c r="D59" s="47"/>
-      <c r="E59" s="32"/>
-      <c r="F59" s="31">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G59" s="36"/>
-      <c r="H59" s="43"/>
-      <c r="I59" s="41"/>
-      <c r="J59" s="37"/>
-      <c r="K59" s="29"/>
-      <c r="L59" s="29"/>
-      <c r="M59" s="29"/>
-      <c r="N59" s="29"/>
-      <c r="O59" s="29"/>
-      <c r="P59" s="44"/>
-    </row>
-    <row r="60" spans="1:16" ht="13">
-      <c r="A60" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B60" s="6"/>
-      <c r="D60" s="47"/>
-      <c r="E60" s="32"/>
-      <c r="F60" s="31">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G60" s="36"/>
-      <c r="H60" s="43"/>
-      <c r="I60" s="41"/>
-      <c r="J60" s="37"/>
-      <c r="P60" s="46"/>
-    </row>
-    <row r="61" spans="1:16" ht="13">
-      <c r="A61" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B61" s="6"/>
-      <c r="C61" s="38"/>
-      <c r="D61" s="47"/>
-      <c r="E61" s="32"/>
-      <c r="F61" s="31">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G61" s="36"/>
-      <c r="H61" s="43"/>
-      <c r="I61" s="41"/>
-      <c r="J61" s="37"/>
-      <c r="K61" s="29"/>
-      <c r="L61" s="29"/>
-      <c r="M61" s="29"/>
-      <c r="N61" s="29"/>
-      <c r="O61" s="29"/>
-      <c r="P61" s="44"/>
-    </row>
-    <row r="62" spans="1:16" ht="13">
-      <c r="A62" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B62" s="6"/>
-      <c r="C62" s="38"/>
-      <c r="D62" s="47"/>
-      <c r="E62" s="32"/>
-      <c r="F62" s="31">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G62" s="36"/>
-      <c r="H62" s="43"/>
-      <c r="I62" s="41"/>
-      <c r="J62" s="37"/>
-      <c r="K62" s="29"/>
-      <c r="L62" s="29"/>
-      <c r="M62" s="29"/>
-      <c r="N62" s="29"/>
-      <c r="O62" s="29"/>
-      <c r="P62" s="46"/>
-    </row>
-    <row r="63" spans="1:16" ht="13">
-      <c r="A63" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B63" s="6"/>
-      <c r="C63" s="38"/>
-      <c r="D63" s="47"/>
-      <c r="E63" s="32"/>
-      <c r="F63" s="31">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G63" s="36"/>
-      <c r="H63" s="43"/>
-      <c r="I63" s="41"/>
-      <c r="J63" s="37"/>
-      <c r="K63" s="29"/>
-      <c r="L63" s="29"/>
-      <c r="M63" s="29"/>
-      <c r="N63" s="29"/>
-      <c r="O63" s="29"/>
-      <c r="P63" s="34"/>
-    </row>
-    <row r="64" spans="1:16" ht="39">
-      <c r="A64" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B64" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="C64" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="D64" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="E64" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="F64" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="G64" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="H64" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="I64" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="J64" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="P64" s="23" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="65" spans="1:16">
-      <c r="A65" s="22"/>
-      <c r="B65" s="22"/>
-      <c r="C65" s="22"/>
-      <c r="D65" s="22"/>
-      <c r="E65" s="22"/>
-      <c r="F65" s="4"/>
-      <c r="G65" s="4"/>
-      <c r="H65" s="4"/>
-      <c r="I65" s="4"/>
-      <c r="J65" s="4"/>
-      <c r="K65" s="4"/>
-      <c r="L65" s="4"/>
-      <c r="M65" s="4"/>
-      <c r="N65" s="4"/>
-      <c r="O65" s="4"/>
-      <c r="P65" s="4"/>
-    </row>
-    <row r="66" spans="1:16" ht="13">
-      <c r="A66" s="11"/>
-      <c r="B66" s="18"/>
-      <c r="C66" s="11"/>
-      <c r="D66" s="12"/>
-      <c r="E66" s="19"/>
-      <c r="F66" s="8"/>
-      <c r="G66" s="28"/>
-      <c r="H66" s="18"/>
-      <c r="I66" s="14"/>
-      <c r="J66" s="35"/>
-      <c r="P66" s="14"/>
-    </row>
-    <row r="67" spans="1:16" ht="13">
-      <c r="A67" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B67" s="6"/>
-      <c r="C67" s="38"/>
-      <c r="D67"/>
-      <c r="E67" s="6"/>
-      <c r="F67" s="31">
-        <f t="shared" ref="F67:F87" si="3">C67*E67</f>
-        <v>0</v>
-      </c>
-      <c r="G67" s="36"/>
-      <c r="H67" s="41"/>
-      <c r="I67" s="41"/>
-      <c r="J67" s="37"/>
-      <c r="K67" s="29"/>
-      <c r="L67" s="29"/>
-      <c r="M67" s="29"/>
-      <c r="N67" s="29"/>
-      <c r="O67" s="29"/>
-      <c r="P67" s="44"/>
-    </row>
-    <row r="68" spans="1:16" ht="13">
-      <c r="A68" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B68" s="6"/>
-      <c r="C68" s="38"/>
-      <c r="D68" s="49"/>
-      <c r="E68" s="32"/>
-      <c r="F68" s="31">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G68" s="36"/>
-      <c r="H68" s="41"/>
-      <c r="I68" s="41"/>
-      <c r="J68" s="37"/>
-      <c r="K68" s="29"/>
-      <c r="L68" s="29"/>
-      <c r="M68" s="29"/>
-      <c r="N68" s="29"/>
-      <c r="O68" s="29"/>
-      <c r="P68" s="46"/>
-    </row>
-    <row r="69" spans="1:16" ht="13">
-      <c r="A69" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B69" s="6"/>
-      <c r="C69" s="38"/>
-      <c r="D69"/>
-      <c r="E69" s="32"/>
-      <c r="F69" s="31">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G69" s="36"/>
-      <c r="H69" s="41"/>
-      <c r="I69" s="41"/>
-      <c r="J69" s="37"/>
-      <c r="K69" s="29"/>
-      <c r="L69" s="29"/>
-      <c r="M69" s="29"/>
-      <c r="N69" s="29"/>
-      <c r="O69" s="29"/>
-      <c r="P69" s="34"/>
-    </row>
-    <row r="70" spans="1:16" ht="13">
-      <c r="A70" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B70" s="6"/>
-      <c r="C70" s="38"/>
-      <c r="D70"/>
-      <c r="E70" s="32"/>
-      <c r="F70" s="31">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G70" s="36"/>
-      <c r="H70" s="41"/>
-      <c r="I70" s="41"/>
-      <c r="J70" s="37"/>
-      <c r="K70" s="29"/>
-      <c r="L70" s="29"/>
-      <c r="M70" s="29"/>
-      <c r="N70" s="29"/>
-      <c r="O70" s="29"/>
-      <c r="P70" s="44"/>
-    </row>
-    <row r="71" spans="1:16" ht="13">
-      <c r="A71" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B71" s="6"/>
-      <c r="D71"/>
-      <c r="E71" s="32"/>
-      <c r="F71" s="31">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G71" s="36"/>
-      <c r="H71" s="41"/>
-      <c r="I71" s="41"/>
-      <c r="J71" s="37"/>
-      <c r="P71" s="46"/>
-    </row>
-    <row r="72" spans="1:16" ht="13">
-      <c r="A72" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B72" s="6"/>
-      <c r="C72" s="38"/>
-      <c r="D72" s="49"/>
-      <c r="E72" s="32"/>
-      <c r="F72" s="31">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G72" s="36"/>
-      <c r="H72" s="43"/>
-      <c r="I72" s="41"/>
-      <c r="J72" s="37"/>
-      <c r="K72" s="29"/>
-      <c r="L72" s="29"/>
-      <c r="M72" s="29"/>
-      <c r="N72" s="29"/>
-      <c r="O72" s="29"/>
-      <c r="P72" s="44"/>
-    </row>
-    <row r="73" spans="1:16" ht="13">
-      <c r="A73" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B73" s="6"/>
-      <c r="C73" s="38"/>
-      <c r="D73"/>
-      <c r="E73" s="32"/>
-      <c r="F73" s="31">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G73" s="36"/>
-      <c r="H73" s="43"/>
-      <c r="I73" s="41"/>
-      <c r="J73" s="37"/>
-      <c r="K73" s="29"/>
-      <c r="L73" s="29"/>
-      <c r="M73" s="29"/>
-      <c r="N73" s="29"/>
-      <c r="O73" s="29"/>
-      <c r="P73" s="46"/>
-    </row>
-    <row r="74" spans="1:16" ht="13">
-      <c r="A74" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B74" s="6"/>
-      <c r="C74" s="38"/>
-      <c r="D74"/>
-      <c r="E74" s="32"/>
-      <c r="F74" s="31">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G74" s="36"/>
-      <c r="H74" s="43"/>
-      <c r="I74" s="41"/>
-      <c r="J74" s="37"/>
-      <c r="K74" s="29"/>
-      <c r="L74" s="29"/>
-      <c r="M74" s="29"/>
-      <c r="N74" s="29"/>
-      <c r="O74" s="29"/>
-      <c r="P74" s="34"/>
-    </row>
-    <row r="75" spans="1:16" ht="13">
-      <c r="A75" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B75" s="6"/>
-      <c r="C75" s="38"/>
-      <c r="D75"/>
-      <c r="E75" s="32"/>
-      <c r="F75" s="31">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G75" s="36"/>
-      <c r="H75" s="43"/>
-      <c r="I75" s="41"/>
-      <c r="J75" s="37"/>
-      <c r="K75" s="29"/>
-      <c r="L75" s="29"/>
-      <c r="M75" s="29"/>
-      <c r="N75" s="29"/>
-      <c r="O75" s="29"/>
-      <c r="P75" s="44"/>
-    </row>
-    <row r="76" spans="1:16" ht="13">
-      <c r="A76" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B76" s="6"/>
-      <c r="D76"/>
-      <c r="E76" s="32"/>
-      <c r="F76" s="31">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G76" s="36"/>
-      <c r="H76" s="43"/>
-      <c r="I76" s="41"/>
-      <c r="J76" s="37"/>
-      <c r="P76" s="46"/>
-    </row>
-    <row r="77" spans="1:16" ht="13">
-      <c r="A77" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B77" s="6"/>
-      <c r="C77" s="38"/>
-      <c r="D77" s="47"/>
-      <c r="E77" s="32"/>
-      <c r="F77" s="31">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G77" s="36"/>
-      <c r="H77" s="43"/>
-      <c r="I77" s="41"/>
-      <c r="J77" s="37"/>
-      <c r="K77" s="29"/>
-      <c r="L77" s="29"/>
-      <c r="M77" s="29"/>
-      <c r="N77" s="29"/>
-      <c r="O77" s="29"/>
-      <c r="P77" s="44"/>
-    </row>
-    <row r="78" spans="1:16" ht="13">
-      <c r="A78" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B78" s="6"/>
-      <c r="C78" s="38"/>
-      <c r="D78" s="47"/>
-      <c r="E78" s="32"/>
-      <c r="F78" s="31">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G78" s="36"/>
-      <c r="H78" s="43"/>
-      <c r="I78" s="41"/>
-      <c r="J78" s="37"/>
-      <c r="K78" s="29"/>
-      <c r="L78" s="29"/>
-      <c r="M78" s="29"/>
-      <c r="N78" s="29"/>
-      <c r="O78" s="29"/>
-      <c r="P78" s="46"/>
-    </row>
-    <row r="79" spans="1:16" ht="13">
-      <c r="A79" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B79" s="6"/>
-      <c r="C79" s="38"/>
-      <c r="D79" s="47"/>
-      <c r="E79" s="32"/>
-      <c r="F79" s="31">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G79" s="36"/>
-      <c r="H79" s="43"/>
-      <c r="I79" s="41"/>
-      <c r="J79" s="37"/>
-      <c r="K79" s="29"/>
-      <c r="L79" s="29"/>
-      <c r="M79" s="29"/>
-      <c r="N79" s="29"/>
-      <c r="O79" s="29"/>
-      <c r="P79" s="34"/>
-    </row>
-    <row r="80" spans="1:16" ht="13">
-      <c r="A80" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B80" s="6"/>
-      <c r="C80" s="38"/>
-      <c r="D80" s="47"/>
-      <c r="E80" s="32"/>
-      <c r="F80" s="31">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G80" s="36"/>
-      <c r="H80" s="43"/>
-      <c r="I80" s="41"/>
-      <c r="J80" s="37"/>
-      <c r="K80" s="29"/>
-      <c r="L80" s="29"/>
-      <c r="M80" s="29"/>
-      <c r="N80" s="29"/>
-      <c r="O80" s="29"/>
-      <c r="P80" s="44"/>
-    </row>
-    <row r="81" spans="1:16" ht="13">
-      <c r="A81" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B81" s="6"/>
-      <c r="D81" s="47"/>
-      <c r="E81" s="32"/>
-      <c r="F81" s="31">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G81" s="36"/>
-      <c r="H81" s="43"/>
-      <c r="I81" s="41"/>
-      <c r="J81" s="37"/>
-      <c r="P81" s="46"/>
-    </row>
-    <row r="82" spans="1:16" ht="13">
-      <c r="A82" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B82" s="6"/>
-      <c r="C82" s="38"/>
-      <c r="D82" s="47"/>
-      <c r="E82" s="32"/>
-      <c r="F82" s="31">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G82" s="36"/>
-      <c r="H82" s="43"/>
-      <c r="I82" s="41"/>
-      <c r="J82" s="37"/>
-      <c r="K82" s="29"/>
-      <c r="L82" s="29"/>
-      <c r="M82" s="29"/>
-      <c r="N82" s="29"/>
-      <c r="O82" s="29"/>
-      <c r="P82" s="44"/>
-    </row>
-    <row r="83" spans="1:16" ht="13">
-      <c r="A83" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B83" s="6"/>
-      <c r="C83" s="38"/>
-      <c r="D83" s="47"/>
-      <c r="E83" s="32"/>
-      <c r="F83" s="31">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G83" s="36"/>
-      <c r="H83" s="43"/>
-      <c r="I83" s="41"/>
-      <c r="J83" s="37"/>
-      <c r="K83" s="29"/>
-      <c r="L83" s="29"/>
-      <c r="M83" s="29"/>
-      <c r="N83" s="29"/>
-      <c r="O83" s="29"/>
-      <c r="P83" s="46"/>
-    </row>
-    <row r="84" spans="1:16" ht="13">
-      <c r="A84" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B84" s="6"/>
-      <c r="C84" s="38"/>
-      <c r="D84" s="47"/>
-      <c r="E84" s="32"/>
-      <c r="F84" s="31">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G84" s="36"/>
-      <c r="H84" s="43"/>
-      <c r="I84" s="41"/>
-      <c r="J84" s="37"/>
-      <c r="K84" s="29"/>
-      <c r="L84" s="29"/>
-      <c r="M84" s="29"/>
-      <c r="N84" s="29"/>
-      <c r="O84" s="29"/>
-      <c r="P84" s="34"/>
-    </row>
-    <row r="85" spans="1:16" ht="13">
-      <c r="A85" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B85" s="6"/>
-      <c r="C85" s="38"/>
-      <c r="D85" s="47"/>
-      <c r="E85" s="32"/>
-      <c r="F85" s="31">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G85" s="36"/>
-      <c r="H85" s="43"/>
-      <c r="I85" s="41"/>
-      <c r="J85" s="37"/>
-      <c r="K85" s="29"/>
-      <c r="L85" s="29"/>
-      <c r="M85" s="29"/>
-      <c r="N85" s="29"/>
-      <c r="O85" s="29"/>
-      <c r="P85" s="44"/>
-    </row>
-    <row r="86" spans="1:16" ht="13">
-      <c r="A86" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B86" s="6"/>
-      <c r="C86" s="38"/>
-      <c r="D86" s="47"/>
-      <c r="E86" s="32"/>
-      <c r="F86" s="31">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G86" s="36"/>
-      <c r="H86" s="43"/>
-      <c r="I86" s="41"/>
-      <c r="J86" s="37"/>
-      <c r="K86" s="29"/>
-      <c r="L86" s="29"/>
-      <c r="M86" s="29"/>
-      <c r="N86" s="29"/>
-      <c r="O86" s="29"/>
-      <c r="P86" s="44"/>
-    </row>
-    <row r="87" spans="1:16" ht="13">
-      <c r="A87" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B87" s="6"/>
-      <c r="D87" s="47"/>
-      <c r="E87" s="32"/>
-      <c r="F87" s="31">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G87" s="36"/>
-      <c r="H87" s="43"/>
-      <c r="I87" s="41"/>
-      <c r="J87" s="37"/>
-      <c r="P87" s="46"/>
-    </row>
-    <row r="88" spans="1:16">
+      <c r="G36" s="35"/>
+      <c r="H36" s="39"/>
+      <c r="I36" s="39"/>
+      <c r="J36" s="36"/>
+      <c r="P36" s="41"/>
+    </row>
+    <row r="37" spans="1:16">
+      <c r="F37" s="16"/>
+    </row>
+    <row r="38" spans="1:16">
+      <c r="F38" s="16"/>
+    </row>
+    <row r="39" spans="1:16">
+      <c r="F39" s="16"/>
+    </row>
+    <row r="40" spans="1:16">
+      <c r="F40" s="16"/>
+    </row>
+    <row r="41" spans="1:16">
+      <c r="F41" s="16"/>
+    </row>
+    <row r="42" spans="1:16">
+      <c r="F42" s="16"/>
+    </row>
+    <row r="43" spans="1:16">
+      <c r="F43" s="16"/>
+    </row>
+    <row r="44" spans="1:16">
+      <c r="F44" s="16"/>
+    </row>
+    <row r="45" spans="1:16">
+      <c r="F45" s="16"/>
+    </row>
+    <row r="46" spans="1:16">
+      <c r="F46" s="16"/>
+    </row>
+    <row r="47" spans="1:16">
+      <c r="F47" s="16"/>
+    </row>
+    <row r="48" spans="1:16">
+      <c r="F48" s="16"/>
+    </row>
+    <row r="49" spans="6:6">
+      <c r="F49" s="16"/>
+    </row>
+    <row r="50" spans="6:6">
+      <c r="F50" s="16"/>
+    </row>
+    <row r="51" spans="6:6">
+      <c r="F51" s="16"/>
+    </row>
+    <row r="52" spans="6:6">
+      <c r="F52" s="16"/>
+    </row>
+    <row r="53" spans="6:6">
+      <c r="F53" s="16"/>
+    </row>
+    <row r="54" spans="6:6">
+      <c r="F54" s="16"/>
+    </row>
+    <row r="55" spans="6:6">
+      <c r="F55" s="16"/>
+    </row>
+    <row r="56" spans="6:6">
+      <c r="F56" s="16"/>
+    </row>
+    <row r="57" spans="6:6">
+      <c r="F57" s="16"/>
+    </row>
+    <row r="58" spans="6:6">
+      <c r="F58" s="16"/>
+    </row>
+    <row r="59" spans="6:6">
+      <c r="F59" s="16"/>
+    </row>
+    <row r="60" spans="6:6">
+      <c r="F60" s="16"/>
+    </row>
+    <row r="61" spans="6:6">
+      <c r="F61" s="16"/>
+    </row>
+    <row r="62" spans="6:6">
+      <c r="F62" s="16"/>
+    </row>
+    <row r="63" spans="6:6">
+      <c r="F63" s="16"/>
+    </row>
+    <row r="64" spans="6:6">
+      <c r="F64" s="16"/>
+    </row>
+    <row r="65" spans="6:6">
+      <c r="F65" s="16"/>
+    </row>
+    <row r="66" spans="6:6">
+      <c r="F66" s="16"/>
+    </row>
+    <row r="67" spans="6:6">
+      <c r="F67" s="16"/>
+    </row>
+    <row r="68" spans="6:6">
+      <c r="F68" s="16"/>
+    </row>
+    <row r="69" spans="6:6">
+      <c r="F69" s="16"/>
+    </row>
+    <row r="70" spans="6:6">
+      <c r="F70" s="16"/>
+    </row>
+    <row r="71" spans="6:6">
+      <c r="F71" s="16"/>
+    </row>
+    <row r="72" spans="6:6">
+      <c r="F72" s="16"/>
+    </row>
+    <row r="73" spans="6:6">
+      <c r="F73" s="16"/>
+    </row>
+    <row r="74" spans="6:6">
+      <c r="F74" s="16"/>
+    </row>
+    <row r="75" spans="6:6">
+      <c r="F75" s="16"/>
+    </row>
+    <row r="76" spans="6:6">
+      <c r="F76" s="16"/>
+    </row>
+    <row r="77" spans="6:6">
+      <c r="F77" s="16"/>
+    </row>
+    <row r="78" spans="6:6">
+      <c r="F78" s="16"/>
+    </row>
+    <row r="79" spans="6:6">
+      <c r="F79" s="16"/>
+    </row>
+    <row r="80" spans="6:6">
+      <c r="F80" s="16"/>
+    </row>
+    <row r="81" spans="6:6">
+      <c r="F81" s="16"/>
+    </row>
+    <row r="82" spans="6:6">
+      <c r="F82" s="16"/>
+    </row>
+    <row r="83" spans="6:6">
+      <c r="F83" s="16"/>
+    </row>
+    <row r="84" spans="6:6">
+      <c r="F84" s="16"/>
+    </row>
+    <row r="85" spans="6:6">
+      <c r="F85" s="16"/>
+    </row>
+    <row r="86" spans="6:6">
+      <c r="F86" s="16"/>
+    </row>
+    <row r="87" spans="6:6">
+      <c r="F87" s="16"/>
+    </row>
+    <row r="88" spans="6:6">
       <c r="F88" s="16"/>
     </row>
-    <row r="89" spans="1:16">
+    <row r="89" spans="6:6">
       <c r="F89" s="16"/>
     </row>
-    <row r="90" spans="1:16">
+    <row r="90" spans="6:6">
       <c r="F90" s="16"/>
     </row>
-    <row r="91" spans="1:16">
+    <row r="91" spans="6:6">
       <c r="F91" s="16"/>
     </row>
-    <row r="92" spans="1:16">
+    <row r="92" spans="6:6">
       <c r="F92" s="16"/>
     </row>
-    <row r="93" spans="1:16">
+    <row r="93" spans="6:6">
       <c r="F93" s="16"/>
     </row>
-    <row r="94" spans="1:16">
+    <row r="94" spans="6:6">
       <c r="F94" s="16"/>
     </row>
-    <row r="95" spans="1:16">
+    <row r="95" spans="6:6">
       <c r="F95" s="16"/>
     </row>
-    <row r="96" spans="1:16">
+    <row r="96" spans="6:6">
       <c r="F96" s="16"/>
     </row>
     <row r="97" spans="6:6">
@@ -7886,159 +6990,6 @@
     </row>
     <row r="1756" spans="6:6">
       <c r="F1756" s="16"/>
-    </row>
-    <row r="1757" spans="6:6">
-      <c r="F1757" s="16"/>
-    </row>
-    <row r="1758" spans="6:6">
-      <c r="F1758" s="16"/>
-    </row>
-    <row r="1759" spans="6:6">
-      <c r="F1759" s="16"/>
-    </row>
-    <row r="1760" spans="6:6">
-      <c r="F1760" s="16"/>
-    </row>
-    <row r="1761" spans="6:6">
-      <c r="F1761" s="16"/>
-    </row>
-    <row r="1762" spans="6:6">
-      <c r="F1762" s="16"/>
-    </row>
-    <row r="1763" spans="6:6">
-      <c r="F1763" s="16"/>
-    </row>
-    <row r="1764" spans="6:6">
-      <c r="F1764" s="16"/>
-    </row>
-    <row r="1765" spans="6:6">
-      <c r="F1765" s="16"/>
-    </row>
-    <row r="1766" spans="6:6">
-      <c r="F1766" s="16"/>
-    </row>
-    <row r="1767" spans="6:6">
-      <c r="F1767" s="16"/>
-    </row>
-    <row r="1768" spans="6:6">
-      <c r="F1768" s="16"/>
-    </row>
-    <row r="1769" spans="6:6">
-      <c r="F1769" s="16"/>
-    </row>
-    <row r="1770" spans="6:6">
-      <c r="F1770" s="16"/>
-    </row>
-    <row r="1771" spans="6:6">
-      <c r="F1771" s="16"/>
-    </row>
-    <row r="1772" spans="6:6">
-      <c r="F1772" s="16"/>
-    </row>
-    <row r="1773" spans="6:6">
-      <c r="F1773" s="16"/>
-    </row>
-    <row r="1774" spans="6:6">
-      <c r="F1774" s="16"/>
-    </row>
-    <row r="1775" spans="6:6">
-      <c r="F1775" s="16"/>
-    </row>
-    <row r="1776" spans="6:6">
-      <c r="F1776" s="16"/>
-    </row>
-    <row r="1777" spans="6:6">
-      <c r="F1777" s="16"/>
-    </row>
-    <row r="1778" spans="6:6">
-      <c r="F1778" s="16"/>
-    </row>
-    <row r="1779" spans="6:6">
-      <c r="F1779" s="16"/>
-    </row>
-    <row r="1780" spans="6:6">
-      <c r="F1780" s="16"/>
-    </row>
-    <row r="1781" spans="6:6">
-      <c r="F1781" s="16"/>
-    </row>
-    <row r="1782" spans="6:6">
-      <c r="F1782" s="16"/>
-    </row>
-    <row r="1783" spans="6:6">
-      <c r="F1783" s="16"/>
-    </row>
-    <row r="1784" spans="6:6">
-      <c r="F1784" s="16"/>
-    </row>
-    <row r="1785" spans="6:6">
-      <c r="F1785" s="16"/>
-    </row>
-    <row r="1786" spans="6:6">
-      <c r="F1786" s="16"/>
-    </row>
-    <row r="1787" spans="6:6">
-      <c r="F1787" s="16"/>
-    </row>
-    <row r="1788" spans="6:6">
-      <c r="F1788" s="16"/>
-    </row>
-    <row r="1789" spans="6:6">
-      <c r="F1789" s="16"/>
-    </row>
-    <row r="1790" spans="6:6">
-      <c r="F1790" s="16"/>
-    </row>
-    <row r="1791" spans="6:6">
-      <c r="F1791" s="16"/>
-    </row>
-    <row r="1792" spans="6:6">
-      <c r="F1792" s="16"/>
-    </row>
-    <row r="1793" spans="6:6">
-      <c r="F1793" s="16"/>
-    </row>
-    <row r="1794" spans="6:6">
-      <c r="F1794" s="16"/>
-    </row>
-    <row r="1795" spans="6:6">
-      <c r="F1795" s="16"/>
-    </row>
-    <row r="1796" spans="6:6">
-      <c r="F1796" s="16"/>
-    </row>
-    <row r="1797" spans="6:6">
-      <c r="F1797" s="16"/>
-    </row>
-    <row r="1798" spans="6:6">
-      <c r="F1798" s="16"/>
-    </row>
-    <row r="1799" spans="6:6">
-      <c r="F1799" s="16"/>
-    </row>
-    <row r="1800" spans="6:6">
-      <c r="F1800" s="16"/>
-    </row>
-    <row r="1801" spans="6:6">
-      <c r="F1801" s="16"/>
-    </row>
-    <row r="1802" spans="6:6">
-      <c r="F1802" s="16"/>
-    </row>
-    <row r="1803" spans="6:6">
-      <c r="F1803" s="16"/>
-    </row>
-    <row r="1804" spans="6:6">
-      <c r="F1804" s="16"/>
-    </row>
-    <row r="1805" spans="6:6">
-      <c r="F1805" s="16"/>
-    </row>
-    <row r="1806" spans="6:6">
-      <c r="F1806" s="16"/>
-    </row>
-    <row r="1807" spans="6:6">
-      <c r="F1807" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>